<commit_message>
fix: supprime la ligne ^short "Commentaire" résiduelle sur note 86e6cea8d4bd67f4f19f9fcae5708bc60056f35d
</commit_message>
<xml_diff>
--- a/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
+++ b/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-29T15:18:50+00:00</t>
+    <t>2026-07-20T14:28:34+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -749,7 +749,7 @@
     <t>Problème (jdv-code-probleme-cisis)</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-code-probleme-cisis|20260420150251</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-code-probleme-cisis|20260619134043</t>
   </si>
   <si>
     <t>Condition.severity</t>
@@ -764,7 +764,7 @@
     <t>Coding of the severity with a terminology is preferred, where possible.</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-severite-observation-cisis|20260420150250</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-severite-observation-cisis|20260619134042</t>
   </si>
   <si>
     <t>&lt; 272141005 |Severities|</t>
@@ -1232,7 +1232,7 @@
     <t>A simple summary of the stage such as "Stage 3". The determination of the stage is disease-specific.</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-health-status-code-cisis|20260420150250</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-health-status-code-cisis|20260619134042</t>
   </si>
   <si>
     <t xml:space="preserve">con-1
@@ -1355,7 +1355,7 @@
 </t>
   </si>
   <si>
-    <t>Commentaire</t>
+    <t>Additional information about the Condition</t>
   </si>
   <si>
     <t>Comment by the one who determined or updated the Problem.</t>
@@ -8307,7 +8307,7 @@
         <v>81</v>
       </c>
       <c r="G56" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H56" t="s" s="2">
         <v>80</v>

</xml_diff>

<commit_message>
fix: remplace le slicing category par un binding direct 4d75978e5491d68b3be5bbc3312cb46fa3229307
</commit_message>
<xml_diff>
--- a/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
+++ b/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2150" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2112" uniqueCount="424">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-20T14:28:34+00:00</t>
+    <t>2026-07-20T14:36:58+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -709,7 +709,7 @@
     <t>Condition.category</t>
   </si>
   <si>
-    <t>Type d'observation</t>
+    <t>Category</t>
   </si>
   <si>
     <t>A category assigned to the condition.</t>
@@ -718,14 +718,7 @@
     <t>The categorization is often highly contextual and may appear poorly differentiated or not very useful in other contexts.</t>
   </si>
   <si>
-    <t>extensible</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/condition-category|4.0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pattern:coding.system}
-</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-code-probleme-cisis|20260619134043</t>
   </si>
   <si>
     <t>&lt; 404684003 |Clinical finding|</t>
@@ -738,18 +731,6 @@
   </si>
   <si>
     <t>FiveWs.class</t>
-  </si>
-  <si>
-    <t>Condition.category:problemeCisis</t>
-  </si>
-  <si>
-    <t>problemeCisis</t>
-  </si>
-  <si>
-    <t>Problème (jdv-code-probleme-cisis)</t>
-  </si>
-  <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-code-probleme-cisis|20260619134043</t>
   </si>
   <si>
     <t>Condition.severity</t>
@@ -844,6 +825,9 @@
   </si>
   <si>
     <t>Only used if not implicit in code found in Condition.code. If the use case requires attributes from the BodySite resource (e.g. to identify and track separately) then use the standard extension [bodySite](http://hl7.org/fhir/R4/extension-bodysite.html).  May be a summary code, or a reference to a very precise definition of the location, or both.</t>
+  </si>
+  <si>
+    <t>extensible</t>
   </si>
   <si>
     <t>http://hl7.org/fhir/ValueSet/body-site|4.0.1</t>
@@ -1677,7 +1661,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP56"/>
+  <dimension ref="A1:AP55"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="39.61328125" customWidth="true" bestFit="true"/>
@@ -1707,7 +1691,7 @@
     <col min="25" max="25" width="60.78515625" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="70.26171875" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.6640625" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
@@ -4064,26 +4048,26 @@
         <v>80</v>
       </c>
       <c r="X20" t="s" s="2">
+        <v>202</v>
+      </c>
+      <c r="Y20" s="2"/>
+      <c r="Z20" t="s" s="2">
         <v>224</v>
       </c>
-      <c r="Y20" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="Z20" t="s" s="2">
-        <v>225</v>
-      </c>
       <c r="AA20" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AB20" t="s" s="2">
-        <v>226</v>
-      </c>
-      <c r="AC20" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="AC20" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="AD20" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE20" t="s" s="2">
-        <v>141</v>
+        <v>80</v>
       </c>
       <c r="AF20" t="s" s="2">
         <v>220</v>
@@ -4104,16 +4088,16 @@
         <v>80</v>
       </c>
       <c r="AL20" t="s" s="2">
+        <v>225</v>
+      </c>
+      <c r="AM20" t="s" s="2">
+        <v>226</v>
+      </c>
+      <c r="AN20" t="s" s="2">
         <v>227</v>
       </c>
-      <c r="AM20" t="s" s="2">
+      <c r="AO20" t="s" s="2">
         <v>228</v>
-      </c>
-      <c r="AN20" t="s" s="2">
-        <v>229</v>
-      </c>
-      <c r="AO20" t="s" s="2">
-        <v>230</v>
       </c>
       <c r="AP20" t="s" s="2">
         <v>80</v>
@@ -4121,14 +4105,12 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>220</v>
-      </c>
-      <c r="C21" t="s" s="2">
-        <v>232</v>
-      </c>
+        <v>229</v>
+      </c>
+      <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
         <v>80</v>
       </c>
@@ -4137,7 +4119,7 @@
         <v>81</v>
       </c>
       <c r="G21" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H21" t="s" s="2">
         <v>80</v>
@@ -4152,13 +4134,13 @@
         <v>198</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="N21" t="s" s="2">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
@@ -4188,7 +4170,7 @@
       </c>
       <c r="Y21" s="2"/>
       <c r="Z21" t="s" s="2">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>80</v>
@@ -4206,13 +4188,13 @@
         <v>80</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH21" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI21" t="s" s="2">
         <v>80</v>
@@ -4224,35 +4206,35 @@
         <v>80</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="AM21" t="s" s="2">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="AN21" t="s" s="2">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="AO21" t="s" s="2">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="AP21" t="s" s="2">
-        <v>80</v>
+        <v>238</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
-        <v>80</v>
+        <v>240</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G22" t="s" s="2">
         <v>92</v>
@@ -4264,21 +4246,21 @@
         <v>80</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K22" t="s" s="2">
         <v>198</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>237</v>
-      </c>
-      <c r="N22" t="s" s="2">
-        <v>238</v>
-      </c>
-      <c r="O22" s="2"/>
+        <v>242</v>
+      </c>
+      <c r="N22" s="2"/>
+      <c r="O22" t="s" s="2">
+        <v>243</v>
+      </c>
       <c r="P22" t="s" s="2">
         <v>80</v>
       </c>
@@ -4302,29 +4284,31 @@
         <v>80</v>
       </c>
       <c r="X22" t="s" s="2">
-        <v>202</v>
-      </c>
-      <c r="Y22" s="2"/>
+        <v>116</v>
+      </c>
+      <c r="Y22" t="s" s="2">
+        <v>244</v>
+      </c>
       <c r="Z22" t="s" s="2">
+        <v>245</v>
+      </c>
+      <c r="AA22" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB22" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC22" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD22" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE22" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF22" t="s" s="2">
         <v>239</v>
-      </c>
-      <c r="AA22" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB22" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC22" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD22" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE22" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF22" t="s" s="2">
-        <v>235</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>81</v>
@@ -4339,41 +4323,41 @@
         <v>104</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>80</v>
+        <v>246</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="AM22" t="s" s="2">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="AO22" t="s" s="2">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="AP22" t="s" s="2">
-        <v>244</v>
+        <v>251</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>246</v>
+        <v>80</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G23" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H23" t="s" s="2">
         <v>80</v>
@@ -4388,15 +4372,15 @@
         <v>198</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="N23" s="2"/>
-      <c r="O23" t="s" s="2">
-        <v>249</v>
-      </c>
+        <v>254</v>
+      </c>
+      <c r="N23" t="s" s="2">
+        <v>255</v>
+      </c>
+      <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>80</v>
       </c>
@@ -4420,13 +4404,11 @@
         <v>80</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="Y23" t="s" s="2">
-        <v>250</v>
-      </c>
+        <v>256</v>
+      </c>
+      <c r="Y23" s="2"/>
       <c r="Z23" t="s" s="2">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>80</v>
@@ -4444,45 +4426,45 @@
         <v>80</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI23" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>104</v>
+        <v>258</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>252</v>
+        <v>80</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>254</v>
+        <v>80</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="AO23" t="s" s="2">
-        <v>256</v>
+        <v>80</v>
       </c>
       <c r="AP23" t="s" s="2">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4493,7 +4475,7 @@
         <v>81</v>
       </c>
       <c r="G24" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H24" t="s" s="2">
         <v>80</v>
@@ -4502,20 +4484,18 @@
         <v>80</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>198</v>
+        <v>263</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>259</v>
+        <v>152</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>260</v>
-      </c>
-      <c r="N24" t="s" s="2">
-        <v>261</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="N24" s="2"/>
       <c r="O24" s="2"/>
       <c r="P24" t="s" s="2">
         <v>80</v>
@@ -4540,11 +4520,13 @@
         <v>80</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>224</v>
-      </c>
-      <c r="Y24" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="Y24" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="Z24" t="s" s="2">
-        <v>262</v>
+        <v>80</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>80</v>
@@ -4562,56 +4544,56 @@
         <v>80</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>258</v>
+        <v>154</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH24" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI24" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>263</v>
+        <v>80</v>
       </c>
       <c r="AK24" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>264</v>
+        <v>80</v>
       </c>
       <c r="AM24" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN24" t="s" s="2">
-        <v>265</v>
+        <v>156</v>
       </c>
       <c r="AO24" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP24" t="s" s="2">
-        <v>266</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>80</v>
+        <v>182</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>80</v>
@@ -4623,15 +4605,17 @@
         <v>80</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>268</v>
+        <v>137</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>152</v>
+        <v>265</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="N25" s="2"/>
+        <v>266</v>
+      </c>
+      <c r="N25" t="s" s="2">
+        <v>185</v>
+      </c>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
         <v>80</v>
@@ -4668,31 +4652,31 @@
         <v>80</v>
       </c>
       <c r="AB25" t="s" s="2">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="AC25" t="s" s="2">
-        <v>80</v>
+        <v>159</v>
       </c>
       <c r="AD25" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE25" t="s" s="2">
-        <v>80</v>
+        <v>141</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ25" t="s" s="2">
-        <v>80</v>
+        <v>143</v>
       </c>
       <c r="AK25" t="s" s="2">
         <v>80</v>
@@ -4715,21 +4699,23 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>269</v>
-      </c>
-      <c r="C26" s="2"/>
+        <v>264</v>
+      </c>
+      <c r="C26" t="s" s="2">
+        <v>268</v>
+      </c>
       <c r="D26" t="s" s="2">
-        <v>182</v>
+        <v>80</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G26" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H26" t="s" s="2">
         <v>80</v>
@@ -4741,7 +4727,7 @@
         <v>80</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>137</v>
+        <v>269</v>
       </c>
       <c r="L26" t="s" s="2">
         <v>270</v>
@@ -4749,9 +4735,7 @@
       <c r="M26" t="s" s="2">
         <v>271</v>
       </c>
-      <c r="N26" t="s" s="2">
-        <v>185</v>
-      </c>
+      <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
         <v>80</v>
@@ -4788,16 +4772,16 @@
         <v>80</v>
       </c>
       <c r="AB26" t="s" s="2">
-        <v>140</v>
+        <v>80</v>
       </c>
       <c r="AC26" t="s" s="2">
-        <v>159</v>
+        <v>80</v>
       </c>
       <c r="AD26" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE26" t="s" s="2">
-        <v>141</v>
+        <v>80</v>
       </c>
       <c r="AF26" t="s" s="2">
         <v>160</v>
@@ -4824,7 +4808,7 @@
         <v>80</v>
       </c>
       <c r="AN26" t="s" s="2">
-        <v>156</v>
+        <v>80</v>
       </c>
       <c r="AO26" t="s" s="2">
         <v>80</v>
@@ -4838,11 +4822,9 @@
         <v>272</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>269</v>
-      </c>
-      <c r="C27" t="s" s="2">
         <v>273</v>
       </c>
+      <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
         <v>80</v>
       </c>
@@ -4863,13 +4845,13 @@
         <v>80</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>274</v>
+        <v>94</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>275</v>
+        <v>152</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>276</v>
+        <v>153</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -4920,19 +4902,19 @@
         <v>80</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI27" t="s" s="2">
-        <v>80</v>
+        <v>155</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>143</v>
+        <v>80</v>
       </c>
       <c r="AK27" t="s" s="2">
         <v>80</v>
@@ -4944,7 +4926,7 @@
         <v>80</v>
       </c>
       <c r="AN27" t="s" s="2">
-        <v>80</v>
+        <v>156</v>
       </c>
       <c r="AO27" t="s" s="2">
         <v>80</v>
@@ -4955,10 +4937,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4969,7 +4951,7 @@
         <v>81</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>80</v>
@@ -4981,13 +4963,13 @@
         <v>80</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>94</v>
+        <v>137</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -5026,31 +5008,31 @@
         <v>80</v>
       </c>
       <c r="AB28" t="s" s="2">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="AC28" t="s" s="2">
-        <v>80</v>
+        <v>159</v>
       </c>
       <c r="AD28" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE28" t="s" s="2">
-        <v>80</v>
+        <v>141</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI28" t="s" s="2">
-        <v>155</v>
+        <v>80</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>80</v>
+        <v>143</v>
       </c>
       <c r="AK28" t="s" s="2">
         <v>80</v>
@@ -5062,7 +5044,7 @@
         <v>80</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>156</v>
+        <v>80</v>
       </c>
       <c r="AO28" t="s" s="2">
         <v>80</v>
@@ -5073,10 +5055,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -5084,10 +5066,10 @@
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>80</v>
@@ -5099,22 +5081,24 @@
         <v>80</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>137</v>
+        <v>106</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>138</v>
+        <v>163</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="N29" s="2"/>
+        <v>164</v>
+      </c>
+      <c r="N29" t="s" s="2">
+        <v>165</v>
+      </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="Q29" s="2"/>
       <c r="R29" t="s" s="2">
-        <v>80</v>
+        <v>278</v>
       </c>
       <c r="S29" t="s" s="2">
         <v>80</v>
@@ -5144,31 +5128,31 @@
         <v>80</v>
       </c>
       <c r="AB29" t="s" s="2">
-        <v>140</v>
+        <v>80</v>
       </c>
       <c r="AC29" t="s" s="2">
-        <v>159</v>
+        <v>80</v>
       </c>
       <c r="AD29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE29" t="s" s="2">
-        <v>141</v>
+        <v>80</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="AG29" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>143</v>
+        <v>80</v>
       </c>
       <c r="AK29" t="s" s="2">
         <v>80</v>
@@ -5180,7 +5164,7 @@
         <v>80</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>80</v>
+        <v>135</v>
       </c>
       <c r="AO29" t="s" s="2">
         <v>80</v>
@@ -5191,10 +5175,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5217,24 +5201,22 @@
         <v>80</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>106</v>
+        <v>281</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>163</v>
+        <v>282</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>164</v>
-      </c>
-      <c r="N30" t="s" s="2">
-        <v>165</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>80</v>
       </c>
       <c r="Q30" s="2"/>
       <c r="R30" t="s" s="2">
-        <v>283</v>
+        <v>80</v>
       </c>
       <c r="S30" t="s" s="2">
         <v>80</v>
@@ -5276,19 +5258,19 @@
         <v>80</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="AG30" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="AH30" t="s" s="2">
         <v>92</v>
       </c>
       <c r="AI30" t="s" s="2">
-        <v>80</v>
+        <v>174</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="AK30" t="s" s="2">
         <v>80</v>
@@ -5311,10 +5293,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5322,10 +5304,10 @@
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H31" t="s" s="2">
         <v>80</v>
@@ -5334,19 +5316,23 @@
         <v>80</v>
       </c>
       <c r="J31" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K31" t="s" s="2">
+        <v>284</v>
+      </c>
+      <c r="L31" t="s" s="2">
+        <v>285</v>
+      </c>
+      <c r="M31" t="s" s="2">
         <v>286</v>
       </c>
-      <c r="L31" t="s" s="2">
+      <c r="N31" t="s" s="2">
         <v>287</v>
       </c>
-      <c r="M31" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
+      <c r="O31" t="s" s="2">
+        <v>288</v>
+      </c>
       <c r="P31" t="s" s="2">
         <v>80</v>
       </c>
@@ -5394,16 +5380,16 @@
         <v>80</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>173</v>
+        <v>289</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI31" t="s" s="2">
-        <v>174</v>
+        <v>80</v>
       </c>
       <c r="AJ31" t="s" s="2">
         <v>104</v>
@@ -5415,10 +5401,10 @@
         <v>80</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>80</v>
+        <v>290</v>
       </c>
       <c r="AN31" t="s" s="2">
-        <v>135</v>
+        <v>291</v>
       </c>
       <c r="AO31" t="s" s="2">
         <v>80</v>
@@ -5429,10 +5415,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5443,7 +5429,7 @@
         <v>81</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H32" t="s" s="2">
         <v>80</v>
@@ -5455,19 +5441,19 @@
         <v>93</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>289</v>
+        <v>263</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="O32" t="s" s="2">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="P32" t="s" s="2">
         <v>80</v>
@@ -5516,13 +5502,13 @@
         <v>80</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI32" t="s" s="2">
         <v>80</v>
@@ -5537,10 +5523,10 @@
         <v>80</v>
       </c>
       <c r="AM32" t="s" s="2">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="AN32" t="s" s="2">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="AO32" t="s" s="2">
         <v>80</v>
@@ -5551,18 +5537,18 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>80</v>
+        <v>301</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G33" t="s" s="2">
         <v>92</v>
@@ -5577,19 +5563,17 @@
         <v>93</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>268</v>
+        <v>302</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>299</v>
-      </c>
-      <c r="N33" t="s" s="2">
-        <v>300</v>
-      </c>
+        <v>304</v>
+      </c>
+      <c r="N33" s="2"/>
       <c r="O33" t="s" s="2">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>80</v>
@@ -5638,10 +5622,10 @@
         <v>80</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="AG33" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="AH33" t="s" s="2">
         <v>92</v>
@@ -5653,19 +5637,19 @@
         <v>104</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>80</v>
+        <v>306</v>
       </c>
       <c r="AL33" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="AN33" t="s" s="2">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="AO33" t="s" s="2">
-        <v>80</v>
+        <v>309</v>
       </c>
       <c r="AP33" t="s" s="2">
         <v>80</v>
@@ -5673,18 +5657,18 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>306</v>
+        <v>80</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G34" t="s" s="2">
         <v>92</v>
@@ -5699,18 +5683,18 @@
         <v>93</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>309</v>
-      </c>
-      <c r="N34" s="2"/>
-      <c r="O34" t="s" s="2">
-        <v>310</v>
-      </c>
+        <v>313</v>
+      </c>
+      <c r="N34" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>80</v>
       </c>
@@ -5758,10 +5742,10 @@
         <v>80</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="AG34" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="AH34" t="s" s="2">
         <v>92</v>
@@ -5773,19 +5757,19 @@
         <v>104</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="AL34" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="AO34" t="s" s="2">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="AP34" t="s" s="2">
         <v>80</v>
@@ -5793,10 +5777,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5804,7 +5788,7 @@
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G35" t="s" s="2">
         <v>92</v>
@@ -5819,16 +5803,16 @@
         <v>93</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5866,19 +5850,17 @@
         <v>80</v>
       </c>
       <c r="AB35" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC35" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>324</v>
+      </c>
+      <c r="AC35" s="2"/>
       <c r="AD35" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE35" t="s" s="2">
-        <v>80</v>
+        <v>325</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>81</v>
@@ -5893,19 +5875,19 @@
         <v>104</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="AN35" t="s" s="2">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="AO35" t="s" s="2">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="AP35" t="s" s="2">
         <v>80</v>
@@ -5913,18 +5895,20 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>324</v>
-      </c>
-      <c r="C36" s="2"/>
+        <v>319</v>
+      </c>
+      <c r="C36" t="s" s="2">
+        <v>331</v>
+      </c>
       <c r="D36" t="s" s="2">
         <v>80</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G36" t="s" s="2">
         <v>92</v>
@@ -5939,16 +5923,16 @@
         <v>93</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>325</v>
+        <v>170</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
@@ -5986,17 +5970,19 @@
         <v>80</v>
       </c>
       <c r="AB36" t="s" s="2">
-        <v>329</v>
-      </c>
-      <c r="AC36" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="AC36" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="AD36" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE36" t="s" s="2">
-        <v>330</v>
+        <v>80</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>81</v>
@@ -6011,19 +5997,19 @@
         <v>104</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="AO36" t="s" s="2">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="AP36" t="s" s="2">
         <v>80</v>
@@ -6031,14 +6017,12 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>324</v>
-      </c>
-      <c r="C37" t="s" s="2">
-        <v>336</v>
-      </c>
+        <v>334</v>
+      </c>
+      <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
         <v>80</v>
       </c>
@@ -6056,19 +6040,19 @@
         <v>80</v>
       </c>
       <c r="J37" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>170</v>
+        <v>320</v>
       </c>
       <c r="L37" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="M37" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="N37" t="s" s="2">
         <v>337</v>
-      </c>
-      <c r="M37" t="s" s="2">
-        <v>338</v>
-      </c>
-      <c r="N37" t="s" s="2">
-        <v>328</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -6106,19 +6090,17 @@
         <v>80</v>
       </c>
       <c r="AB37" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC37" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>324</v>
+      </c>
+      <c r="AC37" s="2"/>
       <c r="AD37" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE37" t="s" s="2">
-        <v>80</v>
+        <v>325</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>324</v>
+        <v>334</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>81</v>
@@ -6127,25 +6109,25 @@
         <v>92</v>
       </c>
       <c r="AI37" t="s" s="2">
-        <v>80</v>
+        <v>338</v>
       </c>
       <c r="AJ37" t="s" s="2">
         <v>104</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>331</v>
+        <v>80</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>332</v>
+        <v>80</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="AO37" t="s" s="2">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="AP37" t="s" s="2">
         <v>80</v>
@@ -6153,12 +6135,14 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>339</v>
-      </c>
-      <c r="C38" s="2"/>
+        <v>334</v>
+      </c>
+      <c r="C38" t="s" s="2">
+        <v>342</v>
+      </c>
       <c r="D38" t="s" s="2">
         <v>80</v>
       </c>
@@ -6179,16 +6163,16 @@
         <v>80</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>325</v>
+        <v>170</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -6226,17 +6210,19 @@
         <v>80</v>
       </c>
       <c r="AB38" t="s" s="2">
-        <v>329</v>
-      </c>
-      <c r="AC38" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="AC38" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="AD38" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE38" t="s" s="2">
-        <v>330</v>
+        <v>80</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>81</v>
@@ -6245,7 +6231,7 @@
         <v>92</v>
       </c>
       <c r="AI38" t="s" s="2">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="AJ38" t="s" s="2">
         <v>104</v>
@@ -6260,10 +6246,10 @@
         <v>80</v>
       </c>
       <c r="AN38" t="s" s="2">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="AO38" t="s" s="2">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="AP38" t="s" s="2">
         <v>80</v>
@@ -6271,14 +6257,12 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>339</v>
-      </c>
-      <c r="C39" t="s" s="2">
-        <v>347</v>
-      </c>
+        <v>345</v>
+      </c>
+      <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
         <v>80</v>
       </c>
@@ -6296,20 +6280,18 @@
         <v>80</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K39" t="s" s="2">
         <v>170</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>349</v>
-      </c>
-      <c r="N39" t="s" s="2">
-        <v>342</v>
-      </c>
+        <v>347</v>
+      </c>
+      <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>80</v>
@@ -6358,7 +6340,7 @@
         <v>80</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>81</v>
@@ -6367,7 +6349,7 @@
         <v>92</v>
       </c>
       <c r="AI39" t="s" s="2">
-        <v>343</v>
+        <v>80</v>
       </c>
       <c r="AJ39" t="s" s="2">
         <v>104</v>
@@ -6379,13 +6361,13 @@
         <v>80</v>
       </c>
       <c r="AM39" t="s" s="2">
-        <v>80</v>
+        <v>348</v>
       </c>
       <c r="AN39" t="s" s="2">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="AO39" t="s" s="2">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="AP39" t="s" s="2">
         <v>80</v>
@@ -6393,10 +6375,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6419,13 +6401,13 @@
         <v>93</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>170</v>
+        <v>352</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -6476,7 +6458,7 @@
         <v>80</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>81</v>
@@ -6497,13 +6479,13 @@
         <v>80</v>
       </c>
       <c r="AM40" t="s" s="2">
-        <v>353</v>
+        <v>80</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="AO40" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="AP40" t="s" s="2">
         <v>80</v>
@@ -6511,10 +6493,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6537,13 +6519,13 @@
         <v>93</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -6594,7 +6576,7 @@
         <v>80</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>81</v>
@@ -6615,13 +6597,13 @@
         <v>80</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>80</v>
+        <v>361</v>
       </c>
       <c r="AN41" t="s" s="2">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="AO41" t="s" s="2">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="AP41" t="s" s="2">
         <v>80</v>
@@ -6629,10 +6611,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6643,7 +6625,7 @@
         <v>81</v>
       </c>
       <c r="G42" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H42" t="s" s="2">
         <v>80</v>
@@ -6652,16 +6634,16 @@
         <v>80</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6712,19 +6694,19 @@
         <v>80</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH42" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI42" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>104</v>
+        <v>368</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>80</v>
@@ -6733,13 +6715,13 @@
         <v>80</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>366</v>
+        <v>80</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="AO42" t="s" s="2">
-        <v>368</v>
+        <v>80</v>
       </c>
       <c r="AP42" t="s" s="2">
         <v>80</v>
@@ -6747,10 +6729,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6761,7 +6743,7 @@
         <v>81</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>80</v>
@@ -6773,13 +6755,13 @@
         <v>80</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>370</v>
+        <v>263</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>371</v>
+        <v>152</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>372</v>
+        <v>153</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -6830,19 +6812,19 @@
         <v>80</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>369</v>
+        <v>154</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI43" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>373</v>
+        <v>80</v>
       </c>
       <c r="AK43" t="s" s="2">
         <v>80</v>
@@ -6854,7 +6836,7 @@
         <v>80</v>
       </c>
       <c r="AN43" t="s" s="2">
-        <v>374</v>
+        <v>156</v>
       </c>
       <c r="AO43" t="s" s="2">
         <v>80</v>
@@ -6865,21 +6847,21 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>80</v>
+        <v>182</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>80</v>
@@ -6891,15 +6873,17 @@
         <v>80</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>268</v>
+        <v>137</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>152</v>
+        <v>265</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="N44" s="2"/>
+        <v>266</v>
+      </c>
+      <c r="N44" t="s" s="2">
+        <v>185</v>
+      </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
         <v>80</v>
@@ -6948,19 +6932,19 @@
         <v>80</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH44" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI44" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ44" t="s" s="2">
-        <v>80</v>
+        <v>143</v>
       </c>
       <c r="AK44" t="s" s="2">
         <v>80</v>
@@ -6983,14 +6967,14 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>182</v>
+        <v>373</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
@@ -7003,24 +6987,26 @@
         <v>80</v>
       </c>
       <c r="I45" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K45" t="s" s="2">
         <v>137</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>270</v>
+        <v>374</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>271</v>
+        <v>375</v>
       </c>
       <c r="N45" t="s" s="2">
         <v>185</v>
       </c>
-      <c r="O45" s="2"/>
+      <c r="O45" t="s" s="2">
+        <v>186</v>
+      </c>
       <c r="P45" t="s" s="2">
         <v>80</v>
       </c>
@@ -7068,7 +7054,7 @@
         <v>80</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>160</v>
+        <v>376</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>81</v>
@@ -7092,7 +7078,7 @@
         <v>80</v>
       </c>
       <c r="AN45" t="s" s="2">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="AO45" t="s" s="2">
         <v>80</v>
@@ -7110,39 +7096,35 @@
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
-        <v>378</v>
+        <v>80</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G46" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H46" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I46" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="J46" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>137</v>
+        <v>198</v>
       </c>
       <c r="L46" t="s" s="2">
+        <v>378</v>
+      </c>
+      <c r="M46" t="s" s="2">
         <v>379</v>
       </c>
-      <c r="M46" t="s" s="2">
-        <v>380</v>
-      </c>
-      <c r="N46" t="s" s="2">
-        <v>185</v>
-      </c>
-      <c r="O46" t="s" s="2">
-        <v>186</v>
-      </c>
+      <c r="N46" s="2"/>
+      <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
         <v>80</v>
       </c>
@@ -7166,13 +7148,11 @@
         <v>80</v>
       </c>
       <c r="X46" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y46" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>202</v>
+      </c>
+      <c r="Y46" s="2"/>
       <c r="Z46" t="s" s="2">
-        <v>80</v>
+        <v>380</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>80</v>
@@ -7190,31 +7170,31 @@
         <v>80</v>
       </c>
       <c r="AF46" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="AG46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH46" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="AI46" t="s" s="2">
         <v>381</v>
       </c>
-      <c r="AG46" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH46" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AI46" t="s" s="2">
-        <v>80</v>
-      </c>
       <c r="AJ46" t="s" s="2">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="AK46" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>80</v>
+        <v>382</v>
       </c>
       <c r="AM46" t="s" s="2">
-        <v>80</v>
+        <v>207</v>
       </c>
       <c r="AN46" t="s" s="2">
-        <v>135</v>
+        <v>249</v>
       </c>
       <c r="AO46" t="s" s="2">
         <v>80</v>
@@ -7225,10 +7205,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7239,7 +7219,7 @@
         <v>81</v>
       </c>
       <c r="G47" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H47" t="s" s="2">
         <v>80</v>
@@ -7251,13 +7231,13 @@
         <v>80</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>198</v>
+        <v>384</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -7284,11 +7264,13 @@
         <v>80</v>
       </c>
       <c r="X47" t="s" s="2">
-        <v>202</v>
-      </c>
-      <c r="Y47" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="Y47" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="Z47" t="s" s="2">
-        <v>385</v>
+        <v>80</v>
       </c>
       <c r="AA47" t="s" s="2">
         <v>80</v>
@@ -7306,16 +7288,16 @@
         <v>80</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH47" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI47" t="s" s="2">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="AJ47" t="s" s="2">
         <v>104</v>
@@ -7324,13 +7306,13 @@
         <v>80</v>
       </c>
       <c r="AL47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN47" t="s" s="2">
         <v>387</v>
-      </c>
-      <c r="AM47" t="s" s="2">
-        <v>207</v>
-      </c>
-      <c r="AN47" t="s" s="2">
-        <v>255</v>
       </c>
       <c r="AO47" t="s" s="2">
         <v>80</v>
@@ -7355,7 +7337,7 @@
         <v>81</v>
       </c>
       <c r="G48" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H48" t="s" s="2">
         <v>80</v>
@@ -7367,13 +7349,13 @@
         <v>80</v>
       </c>
       <c r="K48" t="s" s="2">
+        <v>198</v>
+      </c>
+      <c r="L48" t="s" s="2">
         <v>389</v>
       </c>
-      <c r="L48" t="s" s="2">
+      <c r="M48" t="s" s="2">
         <v>390</v>
-      </c>
-      <c r="M48" t="s" s="2">
-        <v>391</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -7400,13 +7382,13 @@
         <v>80</v>
       </c>
       <c r="X48" t="s" s="2">
-        <v>80</v>
+        <v>391</v>
       </c>
       <c r="Y48" t="s" s="2">
-        <v>80</v>
+        <v>392</v>
       </c>
       <c r="Z48" t="s" s="2">
-        <v>80</v>
+        <v>393</v>
       </c>
       <c r="AA48" t="s" s="2">
         <v>80</v>
@@ -7430,10 +7412,10 @@
         <v>81</v>
       </c>
       <c r="AH48" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI48" t="s" s="2">
-        <v>386</v>
+        <v>80</v>
       </c>
       <c r="AJ48" t="s" s="2">
         <v>104</v>
@@ -7448,7 +7430,7 @@
         <v>80</v>
       </c>
       <c r="AN48" t="s" s="2">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="AO48" t="s" s="2">
         <v>80</v>
@@ -7459,10 +7441,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7473,7 +7455,7 @@
         <v>81</v>
       </c>
       <c r="G49" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H49" t="s" s="2">
         <v>80</v>
@@ -7485,15 +7467,17 @@
         <v>80</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>198</v>
+        <v>365</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>395</v>
-      </c>
-      <c r="N49" s="2"/>
+        <v>397</v>
+      </c>
+      <c r="N49" t="s" s="2">
+        <v>398</v>
+      </c>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
         <v>80</v>
@@ -7518,13 +7502,13 @@
         <v>80</v>
       </c>
       <c r="X49" t="s" s="2">
-        <v>396</v>
+        <v>80</v>
       </c>
       <c r="Y49" t="s" s="2">
-        <v>397</v>
+        <v>80</v>
       </c>
       <c r="Z49" t="s" s="2">
-        <v>398</v>
+        <v>80</v>
       </c>
       <c r="AA49" t="s" s="2">
         <v>80</v>
@@ -7542,19 +7526,19 @@
         <v>80</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH49" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI49" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>104</v>
+        <v>399</v>
       </c>
       <c r="AK49" t="s" s="2">
         <v>80</v>
@@ -7566,7 +7550,7 @@
         <v>80</v>
       </c>
       <c r="AN49" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="AO49" t="s" s="2">
         <v>80</v>
@@ -7577,10 +7561,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7591,7 +7575,7 @@
         <v>81</v>
       </c>
       <c r="G50" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H50" t="s" s="2">
         <v>80</v>
@@ -7603,17 +7587,15 @@
         <v>80</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>370</v>
+        <v>263</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>401</v>
+        <v>152</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>402</v>
-      </c>
-      <c r="N50" t="s" s="2">
-        <v>403</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
         <v>80</v>
@@ -7662,19 +7644,19 @@
         <v>80</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>400</v>
+        <v>154</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH50" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI50" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ50" t="s" s="2">
-        <v>404</v>
+        <v>80</v>
       </c>
       <c r="AK50" t="s" s="2">
         <v>80</v>
@@ -7686,7 +7668,7 @@
         <v>80</v>
       </c>
       <c r="AN50" t="s" s="2">
-        <v>405</v>
+        <v>156</v>
       </c>
       <c r="AO50" t="s" s="2">
         <v>80</v>
@@ -7697,21 +7679,21 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
-        <v>80</v>
+        <v>182</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G51" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H51" t="s" s="2">
         <v>80</v>
@@ -7723,15 +7705,17 @@
         <v>80</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>268</v>
+        <v>137</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>152</v>
+        <v>265</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="N51" s="2"/>
+        <v>266</v>
+      </c>
+      <c r="N51" t="s" s="2">
+        <v>185</v>
+      </c>
       <c r="O51" s="2"/>
       <c r="P51" t="s" s="2">
         <v>80</v>
@@ -7780,19 +7764,19 @@
         <v>80</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH51" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI51" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ51" t="s" s="2">
-        <v>80</v>
+        <v>143</v>
       </c>
       <c r="AK51" t="s" s="2">
         <v>80</v>
@@ -7815,14 +7799,14 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
-        <v>182</v>
+        <v>373</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" t="s" s="2">
@@ -7835,24 +7819,26 @@
         <v>80</v>
       </c>
       <c r="I52" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="J52" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K52" t="s" s="2">
         <v>137</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>270</v>
+        <v>374</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>271</v>
+        <v>375</v>
       </c>
       <c r="N52" t="s" s="2">
         <v>185</v>
       </c>
-      <c r="O52" s="2"/>
+      <c r="O52" t="s" s="2">
+        <v>186</v>
+      </c>
       <c r="P52" t="s" s="2">
         <v>80</v>
       </c>
@@ -7900,7 +7886,7 @@
         <v>80</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>160</v>
+        <v>376</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>81</v>
@@ -7924,7 +7910,7 @@
         <v>80</v>
       </c>
       <c r="AN52" t="s" s="2">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="AO52" t="s" s="2">
         <v>80</v>
@@ -7935,14 +7921,14 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
-        <v>378</v>
+        <v>80</v>
       </c>
       <c r="E53" s="2"/>
       <c r="F53" t="s" s="2">
@@ -7955,26 +7941,22 @@
         <v>80</v>
       </c>
       <c r="I53" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="J53" t="s" s="2">
         <v>93</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>137</v>
+        <v>198</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>379</v>
+        <v>405</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>380</v>
-      </c>
-      <c r="N53" t="s" s="2">
-        <v>185</v>
-      </c>
-      <c r="O53" t="s" s="2">
-        <v>186</v>
-      </c>
+        <v>406</v>
+      </c>
+      <c r="N53" s="2"/>
+      <c r="O53" s="2"/>
       <c r="P53" t="s" s="2">
         <v>80</v>
       </c>
@@ -7998,13 +7980,13 @@
         <v>80</v>
       </c>
       <c r="X53" t="s" s="2">
-        <v>80</v>
+        <v>391</v>
       </c>
       <c r="Y53" t="s" s="2">
-        <v>80</v>
+        <v>407</v>
       </c>
       <c r="Z53" t="s" s="2">
-        <v>80</v>
+        <v>408</v>
       </c>
       <c r="AA53" t="s" s="2">
         <v>80</v>
@@ -8022,7 +8004,7 @@
         <v>80</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>381</v>
+        <v>404</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>81</v>
@@ -8031,25 +8013,25 @@
         <v>82</v>
       </c>
       <c r="AI53" t="s" s="2">
-        <v>80</v>
+        <v>409</v>
       </c>
       <c r="AJ53" t="s" s="2">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="AK53" t="s" s="2">
-        <v>80</v>
+        <v>410</v>
       </c>
       <c r="AL53" t="s" s="2">
-        <v>80</v>
+        <v>225</v>
       </c>
       <c r="AM53" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN53" t="s" s="2">
-        <v>135</v>
+        <v>411</v>
       </c>
       <c r="AO53" t="s" s="2">
-        <v>80</v>
+        <v>412</v>
       </c>
       <c r="AP53" t="s" s="2">
         <v>80</v>
@@ -8057,10 +8039,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -8083,13 +8065,13 @@
         <v>93</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>198</v>
+        <v>414</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -8116,31 +8098,31 @@
         <v>80</v>
       </c>
       <c r="X54" t="s" s="2">
-        <v>396</v>
+        <v>80</v>
       </c>
       <c r="Y54" t="s" s="2">
-        <v>412</v>
+        <v>80</v>
       </c>
       <c r="Z54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE54" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF54" t="s" s="2">
         <v>413</v>
-      </c>
-      <c r="AA54" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB54" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC54" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD54" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE54" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF54" t="s" s="2">
-        <v>409</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>81</v>
@@ -8149,25 +8131,25 @@
         <v>82</v>
       </c>
       <c r="AI54" t="s" s="2">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="AJ54" t="s" s="2">
         <v>104</v>
       </c>
       <c r="AK54" t="s" s="2">
-        <v>415</v>
+        <v>80</v>
       </c>
       <c r="AL54" t="s" s="2">
-        <v>227</v>
+        <v>80</v>
       </c>
       <c r="AM54" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN54" t="s" s="2">
-        <v>416</v>
+        <v>387</v>
       </c>
       <c r="AO54" t="s" s="2">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="AP54" t="s" s="2">
         <v>80</v>
@@ -8175,10 +8157,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8198,16 +8180,16 @@
         <v>80</v>
       </c>
       <c r="J55" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K55" t="s" s="2">
+        <v>418</v>
+      </c>
+      <c r="L55" t="s" s="2">
         <v>419</v>
       </c>
-      <c r="L55" t="s" s="2">
+      <c r="M55" t="s" s="2">
         <v>420</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>421</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -8258,7 +8240,7 @@
         <v>80</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>81</v>
@@ -8267,145 +8249,27 @@
         <v>82</v>
       </c>
       <c r="AI55" t="s" s="2">
-        <v>414</v>
+        <v>80</v>
       </c>
       <c r="AJ55" t="s" s="2">
         <v>104</v>
       </c>
       <c r="AK55" t="s" s="2">
-        <v>80</v>
+        <v>421</v>
       </c>
       <c r="AL55" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM55" t="s" s="2">
-        <v>80</v>
+        <v>422</v>
       </c>
       <c r="AN55" t="s" s="2">
-        <v>392</v>
+        <v>423</v>
       </c>
       <c r="AO55" t="s" s="2">
-        <v>417</v>
+        <v>80</v>
       </c>
       <c r="AP55" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="s" s="2">
-        <v>422</v>
-      </c>
-      <c r="B56" t="s" s="2">
-        <v>422</v>
-      </c>
-      <c r="C56" s="2"/>
-      <c r="D56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E56" s="2"/>
-      <c r="F56" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="G56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="H56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K56" t="s" s="2">
-        <v>423</v>
-      </c>
-      <c r="L56" t="s" s="2">
-        <v>424</v>
-      </c>
-      <c r="M56" t="s" s="2">
-        <v>425</v>
-      </c>
-      <c r="N56" s="2"/>
-      <c r="O56" s="2"/>
-      <c r="P56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q56" s="2"/>
-      <c r="R56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF56" t="s" s="2">
-        <v>422</v>
-      </c>
-      <c r="AG56" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AI56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ56" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="AK56" t="s" s="2">
-        <v>426</v>
-      </c>
-      <c r="AL56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM56" t="s" s="2">
-        <v>427</v>
-      </c>
-      <c r="AN56" t="s" s="2">
-        <v>428</v>
-      </c>
-      <c r="AO56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP56" t="s" s="2">
         <v>80</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: ajoute le JDV FRCoreValueSetConditionCode et son binding sur Condition.code b6bfa1b801bc3512dee61878ad6716f47e61a808
</commit_message>
<xml_diff>
--- a/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
+++ b/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2112" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="423">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-20T14:36:58+00:00</t>
+    <t>2026-07-20T15:18:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -772,7 +772,7 @@
   <si>
     <t>Identification de la condition, du problème ou du diagnostic :
 CIM-10 pour les pathologie  et réactions à une vaccination : Si le problème observé n'est pas trouvé dans la terminologie CIM-10, utiliser le code='R69' display='Causes inconnues et non précisées de morbidité' system='https://smt.esante.gouv.fr/terminologie-cim-10' et décrire le problème sous forme de texte libre
-Réaction allergique : CIM-11 (2.16.840.1.113883.6.347) / Chapitre 04 Maladies du système immunitaire / Bloc Affections allergiques ou d'hyper-sensibilité
+Réaction allergique : CIM-11 / Chapitre 04 Maladies du système immunitaire / Bloc Affections allergiques ou d'hyper-sensibilité
 Si pas de problème ou pas d'information : https://smt.esante.gouv.fr/fhir/ValueSet/jdv-absent-or-unknown-problem-cisis</t>
   </si>
   <si>
@@ -782,10 +782,10 @@
     <t>0..1 to account for primarily narrative only resources.</t>
   </si>
   <si>
-    <t>Valueset to describe the actual problem experienced by the patient</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/uv/ips/ValueSet/problems-uv-ips</t>
+    <t>extensible</t>
+  </si>
+  <si>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-condition-code|2.2.0</t>
   </si>
   <si>
     <t>Event.code</t>
@@ -825,9 +825,6 @@
   </si>
   <si>
     <t>Only used if not implicit in code found in Condition.code. If the use case requires attributes from the BodySite resource (e.g. to identify and track separately) then use the standard extension [bodySite](http://hl7.org/fhir/R4/extension-bodysite.html).  May be a summary code, or a reference to a very precise definition of the location, or both.</t>
-  </si>
-  <si>
-    <t>extensible</t>
   </si>
   <si>
     <t>http://hl7.org/fhir/ValueSet/body-site|4.0.1</t>
@@ -4284,11 +4281,9 @@
         <v>80</v>
       </c>
       <c r="X22" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="Y22" t="s" s="2">
         <v>244</v>
       </c>
+      <c r="Y22" s="2"/>
       <c r="Z22" t="s" s="2">
         <v>245</v>
       </c>
@@ -4404,11 +4399,11 @@
         <v>80</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="Y23" s="2"/>
       <c r="Z23" t="s" s="2">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>80</v>
@@ -4438,33 +4433,33 @@
         <v>80</v>
       </c>
       <c r="AJ23" t="s" s="2">
+        <v>257</v>
+      </c>
+      <c r="AK23" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL23" t="s" s="2">
         <v>258</v>
       </c>
-      <c r="AK23" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL23" t="s" s="2">
+      <c r="AM23" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN23" t="s" s="2">
         <v>259</v>
       </c>
-      <c r="AM23" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN23" t="s" s="2">
+      <c r="AO23" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP23" t="s" s="2">
         <v>260</v>
-      </c>
-      <c r="AO23" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP23" t="s" s="2">
-        <v>261</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4487,7 +4482,7 @@
         <v>80</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="L24" t="s" s="2">
         <v>152</v>
@@ -4579,10 +4574,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4608,10 +4603,10 @@
         <v>137</v>
       </c>
       <c r="L25" t="s" s="2">
+        <v>264</v>
+      </c>
+      <c r="M25" t="s" s="2">
         <v>265</v>
-      </c>
-      <c r="M25" t="s" s="2">
-        <v>266</v>
       </c>
       <c r="N25" t="s" s="2">
         <v>185</v>
@@ -4699,13 +4694,13 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="B26" t="s" s="2">
+        <v>263</v>
+      </c>
+      <c r="C26" t="s" s="2">
         <v>267</v>
-      </c>
-      <c r="B26" t="s" s="2">
-        <v>264</v>
-      </c>
-      <c r="C26" t="s" s="2">
-        <v>268</v>
       </c>
       <c r="D26" t="s" s="2">
         <v>80</v>
@@ -4727,13 +4722,13 @@
         <v>80</v>
       </c>
       <c r="K26" t="s" s="2">
+        <v>268</v>
+      </c>
+      <c r="L26" t="s" s="2">
         <v>269</v>
       </c>
-      <c r="L26" t="s" s="2">
+      <c r="M26" t="s" s="2">
         <v>270</v>
-      </c>
-      <c r="M26" t="s" s="2">
-        <v>271</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
@@ -4819,10 +4814,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
+        <v>271</v>
+      </c>
+      <c r="B27" t="s" s="2">
         <v>272</v>
-      </c>
-      <c r="B27" t="s" s="2">
-        <v>273</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4937,10 +4932,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
+        <v>273</v>
+      </c>
+      <c r="B28" t="s" s="2">
         <v>274</v>
-      </c>
-      <c r="B28" t="s" s="2">
-        <v>275</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -5055,10 +5050,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
+        <v>275</v>
+      </c>
+      <c r="B29" t="s" s="2">
         <v>276</v>
-      </c>
-      <c r="B29" t="s" s="2">
-        <v>277</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -5098,7 +5093,7 @@
       </c>
       <c r="Q29" s="2"/>
       <c r="R29" t="s" s="2">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="S29" t="s" s="2">
         <v>80</v>
@@ -5175,10 +5170,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
+        <v>278</v>
+      </c>
+      <c r="B30" t="s" s="2">
         <v>279</v>
-      </c>
-      <c r="B30" t="s" s="2">
-        <v>280</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5201,10 +5196,10 @@
         <v>80</v>
       </c>
       <c r="K30" t="s" s="2">
+        <v>280</v>
+      </c>
+      <c r="L30" t="s" s="2">
         <v>281</v>
-      </c>
-      <c r="L30" t="s" s="2">
-        <v>282</v>
       </c>
       <c r="M30" t="s" s="2">
         <v>172</v>
@@ -5293,10 +5288,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5319,19 +5314,19 @@
         <v>93</v>
       </c>
       <c r="K31" t="s" s="2">
+        <v>283</v>
+      </c>
+      <c r="L31" t="s" s="2">
         <v>284</v>
       </c>
-      <c r="L31" t="s" s="2">
+      <c r="M31" t="s" s="2">
         <v>285</v>
       </c>
-      <c r="M31" t="s" s="2">
+      <c r="N31" t="s" s="2">
         <v>286</v>
       </c>
-      <c r="N31" t="s" s="2">
+      <c r="O31" t="s" s="2">
         <v>287</v>
-      </c>
-      <c r="O31" t="s" s="2">
-        <v>288</v>
       </c>
       <c r="P31" t="s" s="2">
         <v>80</v>
@@ -5380,7 +5375,7 @@
         <v>80</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>81</v>
@@ -5401,10 +5396,10 @@
         <v>80</v>
       </c>
       <c r="AM31" t="s" s="2">
+        <v>289</v>
+      </c>
+      <c r="AN31" t="s" s="2">
         <v>290</v>
-      </c>
-      <c r="AN31" t="s" s="2">
-        <v>291</v>
       </c>
       <c r="AO31" t="s" s="2">
         <v>80</v>
@@ -5415,10 +5410,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5441,19 +5436,19 @@
         <v>93</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="L32" t="s" s="2">
+        <v>292</v>
+      </c>
+      <c r="M32" t="s" s="2">
         <v>293</v>
       </c>
-      <c r="M32" t="s" s="2">
+      <c r="N32" t="s" s="2">
         <v>294</v>
       </c>
-      <c r="N32" t="s" s="2">
+      <c r="O32" t="s" s="2">
         <v>295</v>
-      </c>
-      <c r="O32" t="s" s="2">
-        <v>296</v>
       </c>
       <c r="P32" t="s" s="2">
         <v>80</v>
@@ -5502,7 +5497,7 @@
         <v>80</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>81</v>
@@ -5523,10 +5518,10 @@
         <v>80</v>
       </c>
       <c r="AM32" t="s" s="2">
+        <v>297</v>
+      </c>
+      <c r="AN32" t="s" s="2">
         <v>298</v>
-      </c>
-      <c r="AN32" t="s" s="2">
-        <v>299</v>
       </c>
       <c r="AO32" t="s" s="2">
         <v>80</v>
@@ -5537,14 +5532,14 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
@@ -5563,17 +5558,17 @@
         <v>93</v>
       </c>
       <c r="K33" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="L33" t="s" s="2">
         <v>302</v>
       </c>
-      <c r="L33" t="s" s="2">
+      <c r="M33" t="s" s="2">
         <v>303</v>
-      </c>
-      <c r="M33" t="s" s="2">
-        <v>304</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" t="s" s="2">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>80</v>
@@ -5622,7 +5617,7 @@
         <v>80</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>92</v>
@@ -5637,19 +5632,19 @@
         <v>104</v>
       </c>
       <c r="AK33" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="AL33" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM33" t="s" s="2">
         <v>306</v>
       </c>
-      <c r="AL33" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM33" t="s" s="2">
+      <c r="AN33" t="s" s="2">
         <v>307</v>
       </c>
-      <c r="AN33" t="s" s="2">
+      <c r="AO33" t="s" s="2">
         <v>308</v>
-      </c>
-      <c r="AO33" t="s" s="2">
-        <v>309</v>
       </c>
       <c r="AP33" t="s" s="2">
         <v>80</v>
@@ -5657,10 +5652,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5683,16 +5678,16 @@
         <v>93</v>
       </c>
       <c r="K34" t="s" s="2">
+        <v>310</v>
+      </c>
+      <c r="L34" t="s" s="2">
         <v>311</v>
       </c>
-      <c r="L34" t="s" s="2">
+      <c r="M34" t="s" s="2">
         <v>312</v>
       </c>
-      <c r="M34" t="s" s="2">
+      <c r="N34" t="s" s="2">
         <v>313</v>
-      </c>
-      <c r="N34" t="s" s="2">
-        <v>314</v>
       </c>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
@@ -5742,7 +5737,7 @@
         <v>80</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>81</v>
@@ -5757,19 +5752,19 @@
         <v>104</v>
       </c>
       <c r="AK34" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="AL34" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM34" t="s" s="2">
         <v>315</v>
       </c>
-      <c r="AL34" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM34" t="s" s="2">
+      <c r="AN34" t="s" s="2">
         <v>316</v>
       </c>
-      <c r="AN34" t="s" s="2">
+      <c r="AO34" t="s" s="2">
         <v>317</v>
-      </c>
-      <c r="AO34" t="s" s="2">
-        <v>318</v>
       </c>
       <c r="AP34" t="s" s="2">
         <v>80</v>
@@ -5777,10 +5772,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5803,16 +5798,16 @@
         <v>93</v>
       </c>
       <c r="K35" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="L35" t="s" s="2">
         <v>320</v>
       </c>
-      <c r="L35" t="s" s="2">
+      <c r="M35" t="s" s="2">
         <v>321</v>
       </c>
-      <c r="M35" t="s" s="2">
+      <c r="N35" t="s" s="2">
         <v>322</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>323</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5850,17 +5845,17 @@
         <v>80</v>
       </c>
       <c r="AB35" t="s" s="2">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="AC35" s="2"/>
       <c r="AD35" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE35" t="s" s="2">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>81</v>
@@ -5875,19 +5870,19 @@
         <v>104</v>
       </c>
       <c r="AK35" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="AL35" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM35" t="s" s="2">
         <v>326</v>
       </c>
-      <c r="AL35" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM35" t="s" s="2">
+      <c r="AN35" t="s" s="2">
         <v>327</v>
       </c>
-      <c r="AN35" t="s" s="2">
+      <c r="AO35" t="s" s="2">
         <v>328</v>
-      </c>
-      <c r="AO35" t="s" s="2">
-        <v>329</v>
       </c>
       <c r="AP35" t="s" s="2">
         <v>80</v>
@@ -5895,13 +5890,13 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="B36" t="s" s="2">
+        <v>318</v>
+      </c>
+      <c r="C36" t="s" s="2">
         <v>330</v>
-      </c>
-      <c r="B36" t="s" s="2">
-        <v>319</v>
-      </c>
-      <c r="C36" t="s" s="2">
-        <v>331</v>
       </c>
       <c r="D36" t="s" s="2">
         <v>80</v>
@@ -5926,13 +5921,13 @@
         <v>170</v>
       </c>
       <c r="L36" t="s" s="2">
+        <v>331</v>
+      </c>
+      <c r="M36" t="s" s="2">
         <v>332</v>
       </c>
-      <c r="M36" t="s" s="2">
-        <v>333</v>
-      </c>
       <c r="N36" t="s" s="2">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
@@ -5982,7 +5977,7 @@
         <v>80</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>81</v>
@@ -5997,19 +5992,19 @@
         <v>104</v>
       </c>
       <c r="AK36" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="AL36" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM36" t="s" s="2">
         <v>326</v>
       </c>
-      <c r="AL36" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM36" t="s" s="2">
+      <c r="AN36" t="s" s="2">
         <v>327</v>
       </c>
-      <c r="AN36" t="s" s="2">
+      <c r="AO36" t="s" s="2">
         <v>328</v>
-      </c>
-      <c r="AO36" t="s" s="2">
-        <v>329</v>
       </c>
       <c r="AP36" t="s" s="2">
         <v>80</v>
@@ -6017,10 +6012,10 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -6043,16 +6038,16 @@
         <v>80</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="L37" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="M37" t="s" s="2">
         <v>335</v>
       </c>
-      <c r="M37" t="s" s="2">
+      <c r="N37" t="s" s="2">
         <v>336</v>
-      </c>
-      <c r="N37" t="s" s="2">
-        <v>337</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -6090,17 +6085,17 @@
         <v>80</v>
       </c>
       <c r="AB37" t="s" s="2">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="AC37" s="2"/>
       <c r="AD37" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE37" t="s" s="2">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>81</v>
@@ -6109,7 +6104,7 @@
         <v>92</v>
       </c>
       <c r="AI37" t="s" s="2">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="AJ37" t="s" s="2">
         <v>104</v>
@@ -6124,10 +6119,10 @@
         <v>80</v>
       </c>
       <c r="AN37" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="AO37" t="s" s="2">
         <v>339</v>
-      </c>
-      <c r="AO37" t="s" s="2">
-        <v>340</v>
       </c>
       <c r="AP37" t="s" s="2">
         <v>80</v>
@@ -6135,13 +6130,13 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="B38" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="C38" t="s" s="2">
         <v>341</v>
-      </c>
-      <c r="B38" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="C38" t="s" s="2">
-        <v>342</v>
       </c>
       <c r="D38" t="s" s="2">
         <v>80</v>
@@ -6166,13 +6161,13 @@
         <v>170</v>
       </c>
       <c r="L38" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="M38" t="s" s="2">
         <v>343</v>
       </c>
-      <c r="M38" t="s" s="2">
-        <v>344</v>
-      </c>
       <c r="N38" t="s" s="2">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -6222,7 +6217,7 @@
         <v>80</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>81</v>
@@ -6231,7 +6226,7 @@
         <v>92</v>
       </c>
       <c r="AI38" t="s" s="2">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="AJ38" t="s" s="2">
         <v>104</v>
@@ -6246,10 +6241,10 @@
         <v>80</v>
       </c>
       <c r="AN38" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="AO38" t="s" s="2">
         <v>339</v>
-      </c>
-      <c r="AO38" t="s" s="2">
-        <v>340</v>
       </c>
       <c r="AP38" t="s" s="2">
         <v>80</v>
@@ -6257,10 +6252,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6286,10 +6281,10 @@
         <v>170</v>
       </c>
       <c r="L39" t="s" s="2">
+        <v>345</v>
+      </c>
+      <c r="M39" t="s" s="2">
         <v>346</v>
-      </c>
-      <c r="M39" t="s" s="2">
-        <v>347</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -6340,7 +6335,7 @@
         <v>80</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>81</v>
@@ -6361,13 +6356,13 @@
         <v>80</v>
       </c>
       <c r="AM39" t="s" s="2">
+        <v>347</v>
+      </c>
+      <c r="AN39" t="s" s="2">
         <v>348</v>
       </c>
-      <c r="AN39" t="s" s="2">
+      <c r="AO39" t="s" s="2">
         <v>349</v>
-      </c>
-      <c r="AO39" t="s" s="2">
-        <v>350</v>
       </c>
       <c r="AP39" t="s" s="2">
         <v>80</v>
@@ -6375,10 +6370,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6401,13 +6396,13 @@
         <v>93</v>
       </c>
       <c r="K40" t="s" s="2">
+        <v>351</v>
+      </c>
+      <c r="L40" t="s" s="2">
         <v>352</v>
       </c>
-      <c r="L40" t="s" s="2">
+      <c r="M40" t="s" s="2">
         <v>353</v>
-      </c>
-      <c r="M40" t="s" s="2">
-        <v>354</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -6458,7 +6453,7 @@
         <v>80</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>81</v>
@@ -6482,10 +6477,10 @@
         <v>80</v>
       </c>
       <c r="AN40" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="AO40" t="s" s="2">
         <v>355</v>
-      </c>
-      <c r="AO40" t="s" s="2">
-        <v>356</v>
       </c>
       <c r="AP40" t="s" s="2">
         <v>80</v>
@@ -6493,10 +6488,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6519,13 +6514,13 @@
         <v>93</v>
       </c>
       <c r="K41" t="s" s="2">
+        <v>357</v>
+      </c>
+      <c r="L41" t="s" s="2">
         <v>358</v>
       </c>
-      <c r="L41" t="s" s="2">
+      <c r="M41" t="s" s="2">
         <v>359</v>
-      </c>
-      <c r="M41" t="s" s="2">
-        <v>360</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -6576,7 +6571,7 @@
         <v>80</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>81</v>
@@ -6597,13 +6592,13 @@
         <v>80</v>
       </c>
       <c r="AM41" t="s" s="2">
+        <v>360</v>
+      </c>
+      <c r="AN41" t="s" s="2">
         <v>361</v>
       </c>
-      <c r="AN41" t="s" s="2">
+      <c r="AO41" t="s" s="2">
         <v>362</v>
-      </c>
-      <c r="AO41" t="s" s="2">
-        <v>363</v>
       </c>
       <c r="AP41" t="s" s="2">
         <v>80</v>
@@ -6611,10 +6606,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6637,13 +6632,13 @@
         <v>80</v>
       </c>
       <c r="K42" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="L42" t="s" s="2">
         <v>365</v>
       </c>
-      <c r="L42" t="s" s="2">
+      <c r="M42" t="s" s="2">
         <v>366</v>
-      </c>
-      <c r="M42" t="s" s="2">
-        <v>367</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6694,7 +6689,7 @@
         <v>80</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>81</v>
@@ -6706,19 +6701,19 @@
         <v>80</v>
       </c>
       <c r="AJ42" t="s" s="2">
+        <v>367</v>
+      </c>
+      <c r="AK42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN42" t="s" s="2">
         <v>368</v>
-      </c>
-      <c r="AK42" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL42" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM42" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN42" t="s" s="2">
-        <v>369</v>
       </c>
       <c r="AO42" t="s" s="2">
         <v>80</v>
@@ -6729,10 +6724,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6755,7 +6750,7 @@
         <v>80</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="L43" t="s" s="2">
         <v>152</v>
@@ -6847,10 +6842,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6876,10 +6871,10 @@
         <v>137</v>
       </c>
       <c r="L44" t="s" s="2">
+        <v>264</v>
+      </c>
+      <c r="M44" t="s" s="2">
         <v>265</v>
-      </c>
-      <c r="M44" t="s" s="2">
-        <v>266</v>
       </c>
       <c r="N44" t="s" s="2">
         <v>185</v>
@@ -6967,14 +6962,14 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
@@ -6996,10 +6991,10 @@
         <v>137</v>
       </c>
       <c r="L45" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="M45" t="s" s="2">
         <v>374</v>
-      </c>
-      <c r="M45" t="s" s="2">
-        <v>375</v>
       </c>
       <c r="N45" t="s" s="2">
         <v>185</v>
@@ -7054,7 +7049,7 @@
         <v>80</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>81</v>
@@ -7089,10 +7084,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7118,10 +7113,10 @@
         <v>198</v>
       </c>
       <c r="L46" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="M46" t="s" s="2">
         <v>378</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>379</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -7152,7 +7147,7 @@
       </c>
       <c r="Y46" s="2"/>
       <c r="Z46" t="s" s="2">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>80</v>
@@ -7170,7 +7165,7 @@
         <v>80</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>81</v>
@@ -7179,7 +7174,7 @@
         <v>92</v>
       </c>
       <c r="AI46" t="s" s="2">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AJ46" t="s" s="2">
         <v>104</v>
@@ -7188,7 +7183,7 @@
         <v>80</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="AM46" t="s" s="2">
         <v>207</v>
@@ -7205,10 +7200,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7231,13 +7226,13 @@
         <v>80</v>
       </c>
       <c r="K47" t="s" s="2">
+        <v>383</v>
+      </c>
+      <c r="L47" t="s" s="2">
         <v>384</v>
       </c>
-      <c r="L47" t="s" s="2">
+      <c r="M47" t="s" s="2">
         <v>385</v>
-      </c>
-      <c r="M47" t="s" s="2">
-        <v>386</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -7288,7 +7283,7 @@
         <v>80</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>81</v>
@@ -7297,7 +7292,7 @@
         <v>82</v>
       </c>
       <c r="AI47" t="s" s="2">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AJ47" t="s" s="2">
         <v>104</v>
@@ -7312,7 +7307,7 @@
         <v>80</v>
       </c>
       <c r="AN47" t="s" s="2">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="AO47" t="s" s="2">
         <v>80</v>
@@ -7323,10 +7318,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7352,10 +7347,10 @@
         <v>198</v>
       </c>
       <c r="L48" t="s" s="2">
+        <v>388</v>
+      </c>
+      <c r="M48" t="s" s="2">
         <v>389</v>
-      </c>
-      <c r="M48" t="s" s="2">
-        <v>390</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -7382,14 +7377,14 @@
         <v>80</v>
       </c>
       <c r="X48" t="s" s="2">
+        <v>390</v>
+      </c>
+      <c r="Y48" t="s" s="2">
         <v>391</v>
       </c>
-      <c r="Y48" t="s" s="2">
+      <c r="Z48" t="s" s="2">
         <v>392</v>
       </c>
-      <c r="Z48" t="s" s="2">
-        <v>393</v>
-      </c>
       <c r="AA48" t="s" s="2">
         <v>80</v>
       </c>
@@ -7406,7 +7401,7 @@
         <v>80</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>81</v>
@@ -7430,7 +7425,7 @@
         <v>80</v>
       </c>
       <c r="AN48" t="s" s="2">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="AO48" t="s" s="2">
         <v>80</v>
@@ -7441,10 +7436,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7467,16 +7462,16 @@
         <v>80</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="L49" t="s" s="2">
+        <v>395</v>
+      </c>
+      <c r="M49" t="s" s="2">
         <v>396</v>
       </c>
-      <c r="M49" t="s" s="2">
+      <c r="N49" t="s" s="2">
         <v>397</v>
-      </c>
-      <c r="N49" t="s" s="2">
-        <v>398</v>
       </c>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
@@ -7526,7 +7521,7 @@
         <v>80</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>81</v>
@@ -7538,19 +7533,19 @@
         <v>80</v>
       </c>
       <c r="AJ49" t="s" s="2">
+        <v>398</v>
+      </c>
+      <c r="AK49" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL49" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM49" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN49" t="s" s="2">
         <v>399</v>
-      </c>
-      <c r="AK49" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL49" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM49" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN49" t="s" s="2">
-        <v>400</v>
       </c>
       <c r="AO49" t="s" s="2">
         <v>80</v>
@@ -7561,10 +7556,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7587,7 +7582,7 @@
         <v>80</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="L50" t="s" s="2">
         <v>152</v>
@@ -7679,10 +7674,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7708,10 +7703,10 @@
         <v>137</v>
       </c>
       <c r="L51" t="s" s="2">
+        <v>264</v>
+      </c>
+      <c r="M51" t="s" s="2">
         <v>265</v>
-      </c>
-      <c r="M51" t="s" s="2">
-        <v>266</v>
       </c>
       <c r="N51" t="s" s="2">
         <v>185</v>
@@ -7799,14 +7794,14 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" t="s" s="2">
@@ -7828,10 +7823,10 @@
         <v>137</v>
       </c>
       <c r="L52" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="M52" t="s" s="2">
         <v>374</v>
-      </c>
-      <c r="M52" t="s" s="2">
-        <v>375</v>
       </c>
       <c r="N52" t="s" s="2">
         <v>185</v>
@@ -7886,7 +7881,7 @@
         <v>80</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>81</v>
@@ -7921,10 +7916,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7950,10 +7945,10 @@
         <v>198</v>
       </c>
       <c r="L53" t="s" s="2">
+        <v>404</v>
+      </c>
+      <c r="M53" t="s" s="2">
         <v>405</v>
-      </c>
-      <c r="M53" t="s" s="2">
-        <v>406</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
@@ -7980,14 +7975,14 @@
         <v>80</v>
       </c>
       <c r="X53" t="s" s="2">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="Y53" t="s" s="2">
+        <v>406</v>
+      </c>
+      <c r="Z53" t="s" s="2">
         <v>407</v>
       </c>
-      <c r="Z53" t="s" s="2">
-        <v>408</v>
-      </c>
       <c r="AA53" t="s" s="2">
         <v>80</v>
       </c>
@@ -8004,7 +7999,7 @@
         <v>80</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>81</v>
@@ -8013,13 +8008,13 @@
         <v>82</v>
       </c>
       <c r="AI53" t="s" s="2">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="AJ53" t="s" s="2">
         <v>104</v>
       </c>
       <c r="AK53" t="s" s="2">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="AL53" t="s" s="2">
         <v>225</v>
@@ -8028,10 +8023,10 @@
         <v>80</v>
       </c>
       <c r="AN53" t="s" s="2">
+        <v>410</v>
+      </c>
+      <c r="AO53" t="s" s="2">
         <v>411</v>
-      </c>
-      <c r="AO53" t="s" s="2">
-        <v>412</v>
       </c>
       <c r="AP53" t="s" s="2">
         <v>80</v>
@@ -8039,10 +8034,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -8065,13 +8060,13 @@
         <v>93</v>
       </c>
       <c r="K54" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="L54" t="s" s="2">
         <v>414</v>
       </c>
-      <c r="L54" t="s" s="2">
+      <c r="M54" t="s" s="2">
         <v>415</v>
-      </c>
-      <c r="M54" t="s" s="2">
-        <v>416</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -8122,7 +8117,7 @@
         <v>80</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>81</v>
@@ -8131,7 +8126,7 @@
         <v>82</v>
       </c>
       <c r="AI54" t="s" s="2">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="AJ54" t="s" s="2">
         <v>104</v>
@@ -8146,10 +8141,10 @@
         <v>80</v>
       </c>
       <c r="AN54" t="s" s="2">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="AO54" t="s" s="2">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="AP54" t="s" s="2">
         <v>80</v>
@@ -8157,10 +8152,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8183,13 +8178,13 @@
         <v>80</v>
       </c>
       <c r="K55" t="s" s="2">
+        <v>417</v>
+      </c>
+      <c r="L55" t="s" s="2">
         <v>418</v>
       </c>
-      <c r="L55" t="s" s="2">
+      <c r="M55" t="s" s="2">
         <v>419</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>420</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -8240,7 +8235,7 @@
         <v>80</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>81</v>
@@ -8255,16 +8250,16 @@
         <v>104</v>
       </c>
       <c r="AK55" t="s" s="2">
+        <v>420</v>
+      </c>
+      <c r="AL55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM55" t="s" s="2">
         <v>421</v>
       </c>
-      <c r="AL55" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM55" t="s" s="2">
+      <c r="AN55" t="s" s="2">
         <v>422</v>
-      </c>
-      <c r="AN55" t="s" s="2">
-        <v>423</v>
       </c>
       <c r="AO55" t="s" s="2">
         <v>80</v>

</xml_diff>

<commit_message>
fix: supprime le binding severity sur FRCoreConditionProfile 3f8b6af5506757644c0af37a41fb16ff851a4471
</commit_message>
<xml_diff>
--- a/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
+++ b/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-20T15:18:49+00:00</t>
+    <t>2026-07-20T15:21:00+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -736,7 +736,7 @@
     <t>Condition.severity</t>
   </si>
   <si>
-    <t>Sévérité</t>
+    <t>Subjective severity of condition</t>
   </si>
   <si>
     <t>A subjective assessment of the severity of the condition as evaluated by the clinician.</t>
@@ -745,7 +745,7 @@
     <t>Coding of the severity with a terminology is preferred, where possible.</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-severite-observation-cisis|20260619134042</t>
+    <t>http://hl7.org/fhir/ValueSet/condition-severity|4.0.1</t>
   </si>
   <si>
     <t>&lt; 272141005 |Severities|</t>
@@ -1686,7 +1686,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="60.78515625" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="70.26171875" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="68.78125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
@@ -4163,7 +4163,7 @@
         <v>80</v>
       </c>
       <c r="X21" t="s" s="2">
-        <v>202</v>
+        <v>116</v>
       </c>
       <c r="Y21" s="2"/>
       <c r="Z21" t="s" s="2">

</xml_diff>

<commit_message>
Update clinicalStatus short description in FSH profile 31f198b49cf11405e341bdb954236a9d6d6bdd2d
</commit_message>
<xml_diff>
--- a/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
+++ b/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="422">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-20T15:21:00+00:00</t>
+    <t>2026-07-20T15:29:23+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -635,7 +635,7 @@
 </t>
   </si>
   <si>
-    <t>Statut du problème</t>
+    <t>Statut clinique du problème</t>
   </si>
   <si>
     <t>The problem status describes the condition of the problem:
@@ -1060,9 +1060,6 @@
   </si>
   <si>
     <t>onsetDateTime</t>
-  </si>
-  <si>
-    <t>Date de début du problème</t>
   </si>
   <si>
     <t>Onset of the symptom, complaint, functional limitation, complication or date of diagnosis. A ‘vague’ date, such as only the year or the month and the year, is permitted.</t>
@@ -5921,10 +5918,10 @@
         <v>170</v>
       </c>
       <c r="L36" t="s" s="2">
+        <v>320</v>
+      </c>
+      <c r="M36" t="s" s="2">
         <v>331</v>
-      </c>
-      <c r="M36" t="s" s="2">
-        <v>332</v>
       </c>
       <c r="N36" t="s" s="2">
         <v>322</v>
@@ -6012,10 +6009,10 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -6041,13 +6038,13 @@
         <v>319</v>
       </c>
       <c r="L37" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="M37" t="s" s="2">
         <v>334</v>
       </c>
-      <c r="M37" t="s" s="2">
+      <c r="N37" t="s" s="2">
         <v>335</v>
-      </c>
-      <c r="N37" t="s" s="2">
-        <v>336</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -6095,7 +6092,7 @@
         <v>324</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>81</v>
@@ -6104,7 +6101,7 @@
         <v>92</v>
       </c>
       <c r="AI37" t="s" s="2">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="AJ37" t="s" s="2">
         <v>104</v>
@@ -6119,10 +6116,10 @@
         <v>80</v>
       </c>
       <c r="AN37" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="AO37" t="s" s="2">
         <v>338</v>
-      </c>
-      <c r="AO37" t="s" s="2">
-        <v>339</v>
       </c>
       <c r="AP37" t="s" s="2">
         <v>80</v>
@@ -6130,13 +6127,13 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="B38" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="C38" t="s" s="2">
         <v>340</v>
-      </c>
-      <c r="B38" t="s" s="2">
-        <v>333</v>
-      </c>
-      <c r="C38" t="s" s="2">
-        <v>341</v>
       </c>
       <c r="D38" t="s" s="2">
         <v>80</v>
@@ -6161,13 +6158,13 @@
         <v>170</v>
       </c>
       <c r="L38" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="M38" t="s" s="2">
         <v>342</v>
       </c>
-      <c r="M38" t="s" s="2">
-        <v>343</v>
-      </c>
       <c r="N38" t="s" s="2">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -6217,7 +6214,7 @@
         <v>80</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>81</v>
@@ -6226,7 +6223,7 @@
         <v>92</v>
       </c>
       <c r="AI38" t="s" s="2">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="AJ38" t="s" s="2">
         <v>104</v>
@@ -6241,10 +6238,10 @@
         <v>80</v>
       </c>
       <c r="AN38" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="AO38" t="s" s="2">
         <v>338</v>
-      </c>
-      <c r="AO38" t="s" s="2">
-        <v>339</v>
       </c>
       <c r="AP38" t="s" s="2">
         <v>80</v>
@@ -6252,10 +6249,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6281,10 +6278,10 @@
         <v>170</v>
       </c>
       <c r="L39" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="M39" t="s" s="2">
         <v>345</v>
-      </c>
-      <c r="M39" t="s" s="2">
-        <v>346</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -6335,7 +6332,7 @@
         <v>80</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>81</v>
@@ -6356,13 +6353,13 @@
         <v>80</v>
       </c>
       <c r="AM39" t="s" s="2">
+        <v>346</v>
+      </c>
+      <c r="AN39" t="s" s="2">
         <v>347</v>
       </c>
-      <c r="AN39" t="s" s="2">
+      <c r="AO39" t="s" s="2">
         <v>348</v>
-      </c>
-      <c r="AO39" t="s" s="2">
-        <v>349</v>
       </c>
       <c r="AP39" t="s" s="2">
         <v>80</v>
@@ -6370,10 +6367,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6396,13 +6393,13 @@
         <v>93</v>
       </c>
       <c r="K40" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="L40" t="s" s="2">
         <v>351</v>
       </c>
-      <c r="L40" t="s" s="2">
+      <c r="M40" t="s" s="2">
         <v>352</v>
-      </c>
-      <c r="M40" t="s" s="2">
-        <v>353</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -6453,7 +6450,7 @@
         <v>80</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>81</v>
@@ -6477,10 +6474,10 @@
         <v>80</v>
       </c>
       <c r="AN40" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="AO40" t="s" s="2">
         <v>354</v>
-      </c>
-      <c r="AO40" t="s" s="2">
-        <v>355</v>
       </c>
       <c r="AP40" t="s" s="2">
         <v>80</v>
@@ -6488,10 +6485,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6514,13 +6511,13 @@
         <v>93</v>
       </c>
       <c r="K41" t="s" s="2">
+        <v>356</v>
+      </c>
+      <c r="L41" t="s" s="2">
         <v>357</v>
       </c>
-      <c r="L41" t="s" s="2">
+      <c r="M41" t="s" s="2">
         <v>358</v>
-      </c>
-      <c r="M41" t="s" s="2">
-        <v>359</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -6571,7 +6568,7 @@
         <v>80</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>81</v>
@@ -6592,13 +6589,13 @@
         <v>80</v>
       </c>
       <c r="AM41" t="s" s="2">
+        <v>359</v>
+      </c>
+      <c r="AN41" t="s" s="2">
         <v>360</v>
       </c>
-      <c r="AN41" t="s" s="2">
+      <c r="AO41" t="s" s="2">
         <v>361</v>
-      </c>
-      <c r="AO41" t="s" s="2">
-        <v>362</v>
       </c>
       <c r="AP41" t="s" s="2">
         <v>80</v>
@@ -6606,10 +6603,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6632,13 +6629,13 @@
         <v>80</v>
       </c>
       <c r="K42" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="L42" t="s" s="2">
         <v>364</v>
       </c>
-      <c r="L42" t="s" s="2">
+      <c r="M42" t="s" s="2">
         <v>365</v>
-      </c>
-      <c r="M42" t="s" s="2">
-        <v>366</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6689,7 +6686,7 @@
         <v>80</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>81</v>
@@ -6701,19 +6698,19 @@
         <v>80</v>
       </c>
       <c r="AJ42" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="AK42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN42" t="s" s="2">
         <v>367</v>
-      </c>
-      <c r="AK42" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL42" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM42" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN42" t="s" s="2">
-        <v>368</v>
       </c>
       <c r="AO42" t="s" s="2">
         <v>80</v>
@@ -6724,10 +6721,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6842,10 +6839,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6962,14 +6959,14 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
@@ -6991,10 +6988,10 @@
         <v>137</v>
       </c>
       <c r="L45" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="M45" t="s" s="2">
         <v>373</v>
-      </c>
-      <c r="M45" t="s" s="2">
-        <v>374</v>
       </c>
       <c r="N45" t="s" s="2">
         <v>185</v>
@@ -7049,7 +7046,7 @@
         <v>80</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>81</v>
@@ -7084,10 +7081,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7113,10 +7110,10 @@
         <v>198</v>
       </c>
       <c r="L46" t="s" s="2">
+        <v>376</v>
+      </c>
+      <c r="M46" t="s" s="2">
         <v>377</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>378</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -7147,7 +7144,7 @@
       </c>
       <c r="Y46" s="2"/>
       <c r="Z46" t="s" s="2">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>80</v>
@@ -7165,7 +7162,7 @@
         <v>80</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>81</v>
@@ -7174,7 +7171,7 @@
         <v>92</v>
       </c>
       <c r="AI46" t="s" s="2">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AJ46" t="s" s="2">
         <v>104</v>
@@ -7183,7 +7180,7 @@
         <v>80</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AM46" t="s" s="2">
         <v>207</v>
@@ -7200,10 +7197,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7226,13 +7223,13 @@
         <v>80</v>
       </c>
       <c r="K47" t="s" s="2">
+        <v>382</v>
+      </c>
+      <c r="L47" t="s" s="2">
         <v>383</v>
       </c>
-      <c r="L47" t="s" s="2">
+      <c r="M47" t="s" s="2">
         <v>384</v>
-      </c>
-      <c r="M47" t="s" s="2">
-        <v>385</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -7283,7 +7280,7 @@
         <v>80</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>81</v>
@@ -7292,7 +7289,7 @@
         <v>82</v>
       </c>
       <c r="AI47" t="s" s="2">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AJ47" t="s" s="2">
         <v>104</v>
@@ -7307,7 +7304,7 @@
         <v>80</v>
       </c>
       <c r="AN47" t="s" s="2">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="AO47" t="s" s="2">
         <v>80</v>
@@ -7318,10 +7315,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7347,10 +7344,10 @@
         <v>198</v>
       </c>
       <c r="L48" t="s" s="2">
+        <v>387</v>
+      </c>
+      <c r="M48" t="s" s="2">
         <v>388</v>
-      </c>
-      <c r="M48" t="s" s="2">
-        <v>389</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -7377,14 +7374,14 @@
         <v>80</v>
       </c>
       <c r="X48" t="s" s="2">
+        <v>389</v>
+      </c>
+      <c r="Y48" t="s" s="2">
         <v>390</v>
       </c>
-      <c r="Y48" t="s" s="2">
+      <c r="Z48" t="s" s="2">
         <v>391</v>
       </c>
-      <c r="Z48" t="s" s="2">
-        <v>392</v>
-      </c>
       <c r="AA48" t="s" s="2">
         <v>80</v>
       </c>
@@ -7401,7 +7398,7 @@
         <v>80</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>81</v>
@@ -7425,7 +7422,7 @@
         <v>80</v>
       </c>
       <c r="AN48" t="s" s="2">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="AO48" t="s" s="2">
         <v>80</v>
@@ -7436,10 +7433,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7462,16 +7459,16 @@
         <v>80</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="L49" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="M49" t="s" s="2">
         <v>395</v>
       </c>
-      <c r="M49" t="s" s="2">
+      <c r="N49" t="s" s="2">
         <v>396</v>
-      </c>
-      <c r="N49" t="s" s="2">
-        <v>397</v>
       </c>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
@@ -7521,7 +7518,7 @@
         <v>80</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>81</v>
@@ -7533,19 +7530,19 @@
         <v>80</v>
       </c>
       <c r="AJ49" t="s" s="2">
+        <v>397</v>
+      </c>
+      <c r="AK49" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL49" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM49" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN49" t="s" s="2">
         <v>398</v>
-      </c>
-      <c r="AK49" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL49" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM49" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN49" t="s" s="2">
-        <v>399</v>
       </c>
       <c r="AO49" t="s" s="2">
         <v>80</v>
@@ -7556,10 +7553,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7674,10 +7671,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7794,14 +7791,14 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" t="s" s="2">
@@ -7823,10 +7820,10 @@
         <v>137</v>
       </c>
       <c r="L52" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="M52" t="s" s="2">
         <v>373</v>
-      </c>
-      <c r="M52" t="s" s="2">
-        <v>374</v>
       </c>
       <c r="N52" t="s" s="2">
         <v>185</v>
@@ -7881,7 +7878,7 @@
         <v>80</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>81</v>
@@ -7916,10 +7913,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7945,10 +7942,10 @@
         <v>198</v>
       </c>
       <c r="L53" t="s" s="2">
+        <v>403</v>
+      </c>
+      <c r="M53" t="s" s="2">
         <v>404</v>
-      </c>
-      <c r="M53" t="s" s="2">
-        <v>405</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
@@ -7975,14 +7972,14 @@
         <v>80</v>
       </c>
       <c r="X53" t="s" s="2">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="Y53" t="s" s="2">
+        <v>405</v>
+      </c>
+      <c r="Z53" t="s" s="2">
         <v>406</v>
       </c>
-      <c r="Z53" t="s" s="2">
-        <v>407</v>
-      </c>
       <c r="AA53" t="s" s="2">
         <v>80</v>
       </c>
@@ -7999,7 +7996,7 @@
         <v>80</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>81</v>
@@ -8008,13 +8005,13 @@
         <v>82</v>
       </c>
       <c r="AI53" t="s" s="2">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="AJ53" t="s" s="2">
         <v>104</v>
       </c>
       <c r="AK53" t="s" s="2">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="AL53" t="s" s="2">
         <v>225</v>
@@ -8023,10 +8020,10 @@
         <v>80</v>
       </c>
       <c r="AN53" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="AO53" t="s" s="2">
         <v>410</v>
-      </c>
-      <c r="AO53" t="s" s="2">
-        <v>411</v>
       </c>
       <c r="AP53" t="s" s="2">
         <v>80</v>
@@ -8034,10 +8031,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -8060,13 +8057,13 @@
         <v>93</v>
       </c>
       <c r="K54" t="s" s="2">
+        <v>412</v>
+      </c>
+      <c r="L54" t="s" s="2">
         <v>413</v>
       </c>
-      <c r="L54" t="s" s="2">
+      <c r="M54" t="s" s="2">
         <v>414</v>
-      </c>
-      <c r="M54" t="s" s="2">
-        <v>415</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -8117,7 +8114,7 @@
         <v>80</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>81</v>
@@ -8126,7 +8123,7 @@
         <v>82</v>
       </c>
       <c r="AI54" t="s" s="2">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="AJ54" t="s" s="2">
         <v>104</v>
@@ -8141,10 +8138,10 @@
         <v>80</v>
       </c>
       <c r="AN54" t="s" s="2">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="AO54" t="s" s="2">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="AP54" t="s" s="2">
         <v>80</v>
@@ -8152,10 +8149,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8178,13 +8175,13 @@
         <v>80</v>
       </c>
       <c r="K55" t="s" s="2">
+        <v>416</v>
+      </c>
+      <c r="L55" t="s" s="2">
         <v>417</v>
       </c>
-      <c r="L55" t="s" s="2">
+      <c r="M55" t="s" s="2">
         <v>418</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>419</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -8235,7 +8232,7 @@
         <v>80</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>81</v>
@@ -8250,16 +8247,16 @@
         <v>104</v>
       </c>
       <c r="AK55" t="s" s="2">
+        <v>419</v>
+      </c>
+      <c r="AL55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM55" t="s" s="2">
         <v>420</v>
       </c>
-      <c r="AL55" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM55" t="s" s="2">
+      <c r="AN55" t="s" s="2">
         <v>421</v>
-      </c>
-      <c r="AN55" t="s" s="2">
-        <v>422</v>
       </c>
       <c r="AO55" t="s" s="2">
         <v>80</v>

</xml_diff>

<commit_message>
Ajoute la slice clinicalStatus sur Condition.stage (FRCoreConditionProfile)
Slice discriminée par un pattern SNOMED CT 260998006 "Clinical staging
(qualifier value)" sur stage.type, avec binding required de
stage.summary vers le JDV jdv-health-status-code-cisis.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> e07114491c38bcf696987aeb7ddcf6b9c54ff209
</commit_message>
<xml_diff>
--- a/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
+++ b/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2373" uniqueCount="435">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-31T14:40:09+00:00</t>
+    <t>2026-09-07T15:17:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -718,7 +718,7 @@
     <t>The categorization is often highly contextual and may appear poorly differentiated or not very useful in other contexts.</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-code-probleme-cisis|20260619134043</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-code-probleme-cisis|20260716085853</t>
   </si>
   <si>
     <t>&lt; 404684003 |Clinical finding|</t>
@@ -1170,6 +1170,10 @@
     <t>Clinical stage or grade of a condition. May include formal severity assessments.</t>
   </si>
   <si>
+    <t xml:space="preserve">pattern:type}
+</t>
+  </si>
+  <si>
     <t>con-1:Stage SHALL have summary or assessment {summary.exists() or assessment.exists()}
 ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}</t>
   </si>
@@ -1203,13 +1207,19 @@
     <t>Condition.stage.summary</t>
   </si>
   <si>
-    <t>Statut clinique du patient</t>
+    <t>Most recent Stage Group</t>
   </si>
   <si>
     <t>A simple summary of the stage such as "Stage 3". The determination of the stage is disease-specific.</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-health-status-code-cisis|20260619134042</t>
+    <t>example</t>
+  </si>
+  <si>
+    <t>Codes describing condition stages (e.g. Cancer stages).</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/condition-stage|4.0.1</t>
   </si>
   <si>
     <t xml:space="preserve">con-1
@@ -1244,9 +1254,6 @@
     <t>The kind of staging, such as pathological or clinical staging.</t>
   </si>
   <si>
-    <t>example</t>
-  </si>
-  <si>
     <t>Codes describing the kind of condition staging (e.g. clinical or pathological).</t>
   </si>
   <si>
@@ -1254,6 +1261,45 @@
   </si>
   <si>
     <t>./inboundRelationship[typeCode=SUBJ].source[classCode=OBS, moodCode=EVN, code="stage type"]</t>
+  </si>
+  <si>
+    <t>Condition.stage:clinicalStatus</t>
+  </si>
+  <si>
+    <t>clinicalStatus</t>
+  </si>
+  <si>
+    <t>Condition.stage:clinicalStatus.id</t>
+  </si>
+  <si>
+    <t>Condition.stage:clinicalStatus.extension</t>
+  </si>
+  <si>
+    <t>Condition.stage:clinicalStatus.modifierExtension</t>
+  </si>
+  <si>
+    <t>Condition.stage:clinicalStatus.summary</t>
+  </si>
+  <si>
+    <t>Statut clinique du patient</t>
+  </si>
+  <si>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-health-status-code-cisis|20260716085852</t>
+  </si>
+  <si>
+    <t>Condition.stage:clinicalStatus.assessment</t>
+  </si>
+  <si>
+    <t>Condition.stage:clinicalStatus.type</t>
+  </si>
+  <si>
+    <t>&lt;valueCodeableConcept xmlns="http://hl7.org/fhir"&gt;
+  &lt;coding&gt;
+    &lt;system value="http://snomed.info/sct"/&gt;
+    &lt;code value="260998006"/&gt;
+    &lt;display value="Clinical staging (qualifier value)"/&gt;
+  &lt;/coding&gt;
+&lt;/valueCodeableConcept&gt;</t>
   </si>
   <si>
     <t>Condition.evidence</t>
@@ -1654,7 +1700,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP55"/>
+  <dimension ref="A1:AP62"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="39.61328125" customWidth="true" bestFit="true"/>
@@ -6673,16 +6719,14 @@
         <v>80</v>
       </c>
       <c r="AB42" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC42" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>366</v>
+      </c>
+      <c r="AC42" s="2"/>
       <c r="AD42" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE42" t="s" s="2">
-        <v>80</v>
+        <v>141</v>
       </c>
       <c r="AF42" t="s" s="2">
         <v>362</v>
@@ -6697,7 +6741,7 @@
         <v>80</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>80</v>
@@ -6709,7 +6753,7 @@
         <v>80</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="AO42" t="s" s="2">
         <v>80</v>
@@ -6720,10 +6764,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6838,10 +6882,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6958,14 +7002,14 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
@@ -6987,10 +7031,10 @@
         <v>137</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="N45" t="s" s="2">
         <v>185</v>
@@ -7045,7 +7089,7 @@
         <v>80</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>81</v>
@@ -7080,10 +7124,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7109,10 +7153,10 @@
         <v>198</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -7139,11 +7183,13 @@
         <v>80</v>
       </c>
       <c r="X46" t="s" s="2">
-        <v>202</v>
-      </c>
-      <c r="Y46" s="2"/>
+        <v>379</v>
+      </c>
+      <c r="Y46" t="s" s="2">
+        <v>380</v>
+      </c>
       <c r="Z46" t="s" s="2">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>80</v>
@@ -7161,7 +7207,7 @@
         <v>80</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>81</v>
@@ -7170,7 +7216,7 @@
         <v>92</v>
       </c>
       <c r="AI46" t="s" s="2">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="AJ46" t="s" s="2">
         <v>104</v>
@@ -7179,7 +7225,7 @@
         <v>80</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="AM46" t="s" s="2">
         <v>207</v>
@@ -7196,10 +7242,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7222,13 +7268,13 @@
         <v>80</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -7279,7 +7325,7 @@
         <v>80</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>81</v>
@@ -7288,7 +7334,7 @@
         <v>82</v>
       </c>
       <c r="AI47" t="s" s="2">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="AJ47" t="s" s="2">
         <v>104</v>
@@ -7303,7 +7349,7 @@
         <v>80</v>
       </c>
       <c r="AN47" t="s" s="2">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="AO47" t="s" s="2">
         <v>80</v>
@@ -7314,10 +7360,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7343,10 +7389,10 @@
         <v>198</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -7373,31 +7419,31 @@
         <v>80</v>
       </c>
       <c r="X48" t="s" s="2">
+        <v>379</v>
+      </c>
+      <c r="Y48" t="s" s="2">
+        <v>392</v>
+      </c>
+      <c r="Z48" t="s" s="2">
+        <v>393</v>
+      </c>
+      <c r="AA48" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB48" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC48" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD48" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE48" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF48" t="s" s="2">
         <v>389</v>
-      </c>
-      <c r="Y48" t="s" s="2">
-        <v>390</v>
-      </c>
-      <c r="Z48" t="s" s="2">
-        <v>391</v>
-      </c>
-      <c r="AA48" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB48" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC48" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD48" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE48" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF48" t="s" s="2">
-        <v>386</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>81</v>
@@ -7421,7 +7467,7 @@
         <v>80</v>
       </c>
       <c r="AN48" t="s" s="2">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="AO48" t="s" s="2">
         <v>80</v>
@@ -7432,12 +7478,14 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>393</v>
-      </c>
-      <c r="C49" s="2"/>
+        <v>362</v>
+      </c>
+      <c r="C49" t="s" s="2">
+        <v>396</v>
+      </c>
       <c r="D49" t="s" s="2">
         <v>80</v>
       </c>
@@ -7446,7 +7494,7 @@
         <v>81</v>
       </c>
       <c r="G49" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H49" t="s" s="2">
         <v>80</v>
@@ -7461,14 +7509,12 @@
         <v>363</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>394</v>
+        <v>364</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>395</v>
-      </c>
-      <c r="N49" t="s" s="2">
-        <v>396</v>
-      </c>
+        <v>365</v>
+      </c>
+      <c r="N49" s="2"/>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
         <v>80</v>
@@ -7517,7 +7563,7 @@
         <v>80</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>393</v>
+        <v>362</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>81</v>
@@ -7529,7 +7575,7 @@
         <v>80</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>397</v>
+        <v>367</v>
       </c>
       <c r="AK49" t="s" s="2">
         <v>80</v>
@@ -7541,7 +7587,7 @@
         <v>80</v>
       </c>
       <c r="AN49" t="s" s="2">
-        <v>398</v>
+        <v>368</v>
       </c>
       <c r="AO49" t="s" s="2">
         <v>80</v>
@@ -7552,10 +7598,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7670,10 +7716,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>400</v>
+        <v>370</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7790,14 +7836,14 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>401</v>
+        <v>371</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" t="s" s="2">
@@ -7819,10 +7865,10 @@
         <v>137</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="N52" t="s" s="2">
         <v>185</v>
@@ -7877,7 +7923,7 @@
         <v>80</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>81</v>
@@ -7912,10 +7958,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>402</v>
+        <v>376</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7926,7 +7972,7 @@
         <v>81</v>
       </c>
       <c r="G53" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H53" t="s" s="2">
         <v>80</v>
@@ -7935,16 +7981,16 @@
         <v>80</v>
       </c>
       <c r="J53" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K53" t="s" s="2">
         <v>198</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>404</v>
+        <v>378</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
@@ -7971,13 +8017,11 @@
         <v>80</v>
       </c>
       <c r="X53" t="s" s="2">
-        <v>389</v>
-      </c>
-      <c r="Y53" t="s" s="2">
-        <v>405</v>
-      </c>
+        <v>202</v>
+      </c>
+      <c r="Y53" s="2"/>
       <c r="Z53" t="s" s="2">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="AA53" t="s" s="2">
         <v>80</v>
@@ -7995,34 +8039,34 @@
         <v>80</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>402</v>
+        <v>376</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH53" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI53" t="s" s="2">
-        <v>407</v>
+        <v>382</v>
       </c>
       <c r="AJ53" t="s" s="2">
         <v>104</v>
       </c>
       <c r="AK53" t="s" s="2">
-        <v>408</v>
+        <v>80</v>
       </c>
       <c r="AL53" t="s" s="2">
-        <v>225</v>
+        <v>383</v>
       </c>
       <c r="AM53" t="s" s="2">
-        <v>80</v>
+        <v>207</v>
       </c>
       <c r="AN53" t="s" s="2">
-        <v>409</v>
+        <v>249</v>
       </c>
       <c r="AO53" t="s" s="2">
-        <v>410</v>
+        <v>80</v>
       </c>
       <c r="AP53" t="s" s="2">
         <v>80</v>
@@ -8030,10 +8074,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>411</v>
+        <v>403</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>411</v>
+        <v>384</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -8053,16 +8097,16 @@
         <v>80</v>
       </c>
       <c r="J54" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>412</v>
+        <v>385</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>413</v>
+        <v>386</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>414</v>
+        <v>387</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -8113,7 +8157,7 @@
         <v>80</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>411</v>
+        <v>384</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>81</v>
@@ -8122,7 +8166,7 @@
         <v>82</v>
       </c>
       <c r="AI54" t="s" s="2">
-        <v>407</v>
+        <v>382</v>
       </c>
       <c r="AJ54" t="s" s="2">
         <v>104</v>
@@ -8137,10 +8181,10 @@
         <v>80</v>
       </c>
       <c r="AN54" t="s" s="2">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="AO54" t="s" s="2">
-        <v>410</v>
+        <v>80</v>
       </c>
       <c r="AP54" t="s" s="2">
         <v>80</v>
@@ -8148,10 +8192,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>415</v>
+        <v>404</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>415</v>
+        <v>389</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8159,10 +8203,10 @@
       </c>
       <c r="E55" s="2"/>
       <c r="F55" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G55" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H55" t="s" s="2">
         <v>80</v>
@@ -8174,13 +8218,13 @@
         <v>80</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>416</v>
+        <v>198</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>417</v>
+        <v>390</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>418</v>
+        <v>391</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -8192,7 +8236,7 @@
         <v>80</v>
       </c>
       <c r="S55" t="s" s="2">
-        <v>80</v>
+        <v>405</v>
       </c>
       <c r="T55" t="s" s="2">
         <v>80</v>
@@ -8207,13 +8251,13 @@
         <v>80</v>
       </c>
       <c r="X55" t="s" s="2">
-        <v>80</v>
+        <v>379</v>
       </c>
       <c r="Y55" t="s" s="2">
-        <v>80</v>
+        <v>392</v>
       </c>
       <c r="Z55" t="s" s="2">
-        <v>80</v>
+        <v>393</v>
       </c>
       <c r="AA55" t="s" s="2">
         <v>80</v>
@@ -8231,13 +8275,13 @@
         <v>80</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>415</v>
+        <v>389</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH55" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI55" t="s" s="2">
         <v>80</v>
@@ -8246,21 +8290,855 @@
         <v>104</v>
       </c>
       <c r="AK55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN55" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="AO55" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP55" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="2">
+        <v>406</v>
+      </c>
+      <c r="B56" t="s" s="2">
+        <v>406</v>
+      </c>
+      <c r="C56" s="2"/>
+      <c r="D56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E56" s="2"/>
+      <c r="F56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G56" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K56" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="L56" t="s" s="2">
+        <v>407</v>
+      </c>
+      <c r="M56" t="s" s="2">
+        <v>408</v>
+      </c>
+      <c r="N56" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="O56" s="2"/>
+      <c r="P56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q56" s="2"/>
+      <c r="R56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF56" t="s" s="2">
+        <v>406</v>
+      </c>
+      <c r="AG56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH56" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ56" t="s" s="2">
+        <v>410</v>
+      </c>
+      <c r="AK56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN56" t="s" s="2">
+        <v>411</v>
+      </c>
+      <c r="AO56" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP56" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="2">
+        <v>412</v>
+      </c>
+      <c r="B57" t="s" s="2">
+        <v>412</v>
+      </c>
+      <c r="C57" s="2"/>
+      <c r="D57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E57" s="2"/>
+      <c r="F57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G57" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="H57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K57" t="s" s="2">
+        <v>262</v>
+      </c>
+      <c r="L57" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="M57" t="s" s="2">
+        <v>153</v>
+      </c>
+      <c r="N57" s="2"/>
+      <c r="O57" s="2"/>
+      <c r="P57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q57" s="2"/>
+      <c r="R57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF57" t="s" s="2">
+        <v>154</v>
+      </c>
+      <c r="AG57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH57" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="AI57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AK57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN57" t="s" s="2">
+        <v>156</v>
+      </c>
+      <c r="AO57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP57" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="B58" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="C58" s="2"/>
+      <c r="D58" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="E58" s="2"/>
+      <c r="F58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G58" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K58" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="L58" t="s" s="2">
+        <v>264</v>
+      </c>
+      <c r="M58" t="s" s="2">
+        <v>265</v>
+      </c>
+      <c r="N58" t="s" s="2">
+        <v>185</v>
+      </c>
+      <c r="O58" s="2"/>
+      <c r="P58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q58" s="2"/>
+      <c r="R58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF58" t="s" s="2">
+        <v>160</v>
+      </c>
+      <c r="AG58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH58" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ58" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="AK58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN58" t="s" s="2">
+        <v>156</v>
+      </c>
+      <c r="AO58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP58" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="2">
+        <v>414</v>
+      </c>
+      <c r="B59" t="s" s="2">
+        <v>414</v>
+      </c>
+      <c r="C59" s="2"/>
+      <c r="D59" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="E59" s="2"/>
+      <c r="F59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G59" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I59" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="J59" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="K59" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="L59" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="M59" t="s" s="2">
+        <v>374</v>
+      </c>
+      <c r="N59" t="s" s="2">
+        <v>185</v>
+      </c>
+      <c r="O59" t="s" s="2">
+        <v>186</v>
+      </c>
+      <c r="P59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q59" s="2"/>
+      <c r="R59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF59" t="s" s="2">
+        <v>375</v>
+      </c>
+      <c r="AG59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH59" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ59" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="AK59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN59" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="AO59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP59" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="B60" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="C60" s="2"/>
+      <c r="D60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E60" s="2"/>
+      <c r="F60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G60" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J60" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="K60" t="s" s="2">
+        <v>198</v>
+      </c>
+      <c r="L60" t="s" s="2">
+        <v>416</v>
+      </c>
+      <c r="M60" t="s" s="2">
+        <v>417</v>
+      </c>
+      <c r="N60" s="2"/>
+      <c r="O60" s="2"/>
+      <c r="P60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q60" s="2"/>
+      <c r="R60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X60" t="s" s="2">
+        <v>379</v>
+      </c>
+      <c r="Y60" t="s" s="2">
+        <v>418</v>
+      </c>
+      <c r="Z60" t="s" s="2">
         <v>419</v>
       </c>
-      <c r="AL55" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM55" t="s" s="2">
+      <c r="AA60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF60" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="AG60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH60" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI60" t="s" s="2">
         <v>420</v>
       </c>
-      <c r="AN55" t="s" s="2">
+      <c r="AJ60" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK60" t="s" s="2">
         <v>421</v>
       </c>
-      <c r="AO55" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP55" t="s" s="2">
+      <c r="AL60" t="s" s="2">
+        <v>225</v>
+      </c>
+      <c r="AM60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN60" t="s" s="2">
+        <v>422</v>
+      </c>
+      <c r="AO60" t="s" s="2">
+        <v>423</v>
+      </c>
+      <c r="AP60" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s" s="2">
+        <v>424</v>
+      </c>
+      <c r="B61" t="s" s="2">
+        <v>424</v>
+      </c>
+      <c r="C61" s="2"/>
+      <c r="D61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E61" s="2"/>
+      <c r="F61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G61" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J61" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="K61" t="s" s="2">
+        <v>425</v>
+      </c>
+      <c r="L61" t="s" s="2">
+        <v>426</v>
+      </c>
+      <c r="M61" t="s" s="2">
+        <v>427</v>
+      </c>
+      <c r="N61" s="2"/>
+      <c r="O61" s="2"/>
+      <c r="P61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q61" s="2"/>
+      <c r="R61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF61" t="s" s="2">
+        <v>424</v>
+      </c>
+      <c r="AG61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH61" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI61" t="s" s="2">
+        <v>420</v>
+      </c>
+      <c r="AJ61" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN61" t="s" s="2">
+        <v>388</v>
+      </c>
+      <c r="AO61" t="s" s="2">
+        <v>423</v>
+      </c>
+      <c r="AP61" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s" s="2">
+        <v>428</v>
+      </c>
+      <c r="B62" t="s" s="2">
+        <v>428</v>
+      </c>
+      <c r="C62" s="2"/>
+      <c r="D62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E62" s="2"/>
+      <c r="F62" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G62" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K62" t="s" s="2">
+        <v>429</v>
+      </c>
+      <c r="L62" t="s" s="2">
+        <v>430</v>
+      </c>
+      <c r="M62" t="s" s="2">
+        <v>431</v>
+      </c>
+      <c r="N62" s="2"/>
+      <c r="O62" s="2"/>
+      <c r="P62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q62" s="2"/>
+      <c r="R62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF62" t="s" s="2">
+        <v>428</v>
+      </c>
+      <c r="AG62" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH62" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ62" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK62" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="AL62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM62" t="s" s="2">
+        <v>433</v>
+      </c>
+      <c r="AN62" t="s" s="2">
+        <v>434</v>
+      </c>
+      <c r="AO62" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP62" t="s" s="2">
         <v>80</v>
       </c>
     </row>

</xml_diff>